<commit_message>
Expand cashflow template to 30 project rows per block
Grows the income and expense blocks from 9 and 18 rows to 30 each, so more
project / cost-center lines fit without inserting rows by hand.

- Generator is now parameterized: row grid derives from block sizes, and
  --source carries labels and entered monthly values over from an earlier
  version of the workbook by locating its section markers
- All sums, KPI rows, cumulative cashflow, overview links and charts are
  rebuilt against the new grid

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USZ2QFd3neqnzoYuSHpCqM
</commit_message>
<xml_diff>
--- a/deliverables/cashflow/Cashflow_SmartInfra_IoT_DusL_Plus_Autostrom_2026_2027.xlsx
+++ b/deliverables/cashflow/Cashflow_SmartInfra_IoT_DusL_Plus_Autostrom_2026_2027.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Übersicht" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Cashflow!$A$1:$W$53</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$A:$B,Cashflow!$7:$7</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$7:$7,Cashflow!$A:$B</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Cashflow!$A$1:$W$85</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$A:$B,Cashflow!$6:$6</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$6:$6,Cashflow!$A:$B</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="64">
   <si>
     <t xml:space="preserve">Cashflow-Planung</t>
   </si>
@@ -34,9 +34,6 @@
     <t xml:space="preserve">Bereich:  SmartInfra / IoT-Büro</t>
   </si>
   <si>
-    <t xml:space="preserve">Projekt:  DusL Plus Autostrom</t>
-  </si>
-  <si>
     <t xml:space="preserve">Zeitraum:  Juli 2026 – Dezember 2027  (18 Monate, monatliche Granularität)</t>
   </si>
   <si>
@@ -115,19 +112,22 @@
     <t xml:space="preserve">1  EINNAHMEN</t>
   </si>
   <si>
-    <t xml:space="preserve">Projektumsätze</t>
+    <t xml:space="preserve">87004006 - LKW / Autostrom+</t>
   </si>
   <si>
     <t xml:space="preserve">Einnahmen</t>
   </si>
   <si>
-    <t xml:space="preserve">Dienstleistungen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hardware / IoT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sonstige Einnahmen</t>
+    <t xml:space="preserve">87004006 - PKW / Autostrom+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87105004 - HanseWerk Natur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87001009 - Stadtwerke Husum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85309000 - Bereichskostenstelle EDM</t>
   </si>
   <si>
     <t xml:space="preserve">Summe Einnahmen</t>
@@ -136,42 +136,9 @@
     <t xml:space="preserve">2  AUSGABEN</t>
   </si>
   <si>
-    <t xml:space="preserve">Personalkosten</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ausgaben</t>
   </si>
   <si>
-    <t xml:space="preserve">Hardware / Sensorik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gateways / Kommunikationstechnik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIM / Mobilfunk / Connectivity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Software / Lizenzen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cloud / Hosting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fremdleistungen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Installation / Montage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dienstreisen / Fahrtkosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Büro / Betriebsmittel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sonstige Kosten</t>
-  </si>
-  <si>
     <t xml:space="preserve">Summe Ausgaben</t>
   </si>
   <si>
@@ -202,7 +169,7 @@
     <t xml:space="preserve">Beispielformat einer Eingabe:  1234,50  →  Anzeige 1.234,50 €   (Ausgaben werden als positive Beträge erfasst)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zusätzliche Zeilen: innerhalb der Blöcke Zeile 9–17 (Einnahmen) bzw. 21–38 (Ausgaben) einfügen – alle Summen erweitern sich automatisch.</t>
+    <t xml:space="preserve">Freie Projektzeilen: Einnahmen Zeile 8–37, Ausgaben Zeile 41–70. Werden noch mehr Zeilen benötigt, innerhalb dieser Blöcke einfügen – alle Summen erweitern sich automatisch.</t>
   </si>
   <si>
     <t xml:space="preserve">Übersicht Cashflow – DusL Plus Autostrom</t>
@@ -796,7 +763,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Cashflow!A42</c:f>
+              <c:f>Cashflow!A74</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -841,7 +808,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Cashflow!$C$7:$T$7</c:f>
+              <c:f>Cashflow!$C$6:$T$6</c:f>
               <c:strCache>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
@@ -903,7 +870,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Cashflow!$B$42:$T$42</c:f>
+              <c:f>Cashflow!$B$74:$T$74</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\–</c:formatCode>
                 <c:ptCount val="19"/>
@@ -917,16 +884,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>20000</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>16500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>20000</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -970,7 +937,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Cashflow!A43</c:f>
+              <c:f>Cashflow!A75</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1015,7 +982,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Cashflow!$C$7:$T$7</c:f>
+              <c:f>Cashflow!$C$6:$T$6</c:f>
               <c:strCache>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
@@ -1077,7 +1044,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Cashflow!$B$43:$T$43</c:f>
+              <c:f>Cashflow!$B$75:$T$75</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\–</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1091,7 +1058,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1100,7 +1067,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1141,11 +1108,11 @@
         </c:ser>
         <c:gapWidth val="40"/>
         <c:overlap val="0"/>
-        <c:axId val="60398517"/>
-        <c:axId val="49431024"/>
+        <c:axId val="53981401"/>
+        <c:axId val="40458638"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60398517"/>
+        <c:axId val="53981401"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1177,7 +1144,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49431024"/>
+        <c:crossAx val="40458638"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1185,7 +1152,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49431024"/>
+        <c:axId val="40458638"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1261,7 +1228,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60398517"/>
+        <c:crossAx val="53981401"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1362,7 +1329,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Cashflow!A44</c:f>
+              <c:f>Cashflow!A76</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1412,7 +1379,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Cashflow!$C$7:$T$7</c:f>
+              <c:f>Cashflow!$C$6:$T$6</c:f>
               <c:strCache>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
@@ -1474,7 +1441,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Cashflow!$B$44:$T$44</c:f>
+              <c:f>Cashflow!$B$76:$T$76</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\–</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1488,16 +1455,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>16500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1542,7 +1509,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Cashflow!A45</c:f>
+              <c:f>Cashflow!A77</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1593,7 +1560,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Cashflow!$C$7:$T$7</c:f>
+              <c:f>Cashflow!$C$6:$T$6</c:f>
               <c:strCache>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
@@ -1655,7 +1622,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Cashflow!$B$45:$T$45</c:f>
+              <c:f>Cashflow!$B$77:$T$77</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00" €";[RED]\-#,##0.00" €";\–</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1669,49 +1636,49 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>21500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1726,11 +1693,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="93676766"/>
-        <c:axId val="82460781"/>
+        <c:axId val="12831196"/>
+        <c:axId val="55401202"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="93676766"/>
+        <c:axId val="12831196"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1762,7 +1729,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82460781"/>
+        <c:crossAx val="55401202"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1770,7 +1737,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82460781"/>
+        <c:axId val="55401202"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1846,7 +1813,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93676766"/>
+        <c:crossAx val="12831196"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2143,7 +2110,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:W53"/>
+  <dimension ref="A1:W85"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -2168,127 +2135,164 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="K6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="N6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="P6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="5" t="s">
+      <c r="Q6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="Q7" s="5" t="s">
+      <c r="R6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="S6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="T6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="5" t="s">
+      <c r="U6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="U7" s="5" t="s">
+      <c r="V6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="5" t="s">
+      <c r="W6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="5" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="7"/>
-      <c r="U8" s="7"/>
-      <c r="V8" s="7"/>
-      <c r="W8" s="7"/>
+      <c r="B8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="11" t="n">
+        <f aca="false">SUM(C8:H8)</f>
+        <v>0</v>
+      </c>
+      <c r="V8" s="11" t="n">
+        <f aca="false">SUM(I8:T8)</f>
+        <v>0</v>
+      </c>
+      <c r="W8" s="12" t="n">
+        <f aca="false">SUM(C8:T8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>30</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
+      <c r="F9" s="10" t="n">
+        <v>20000</v>
+      </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
+      <c r="I9" s="10" t="n">
+        <v>20000</v>
+      </c>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
       <c r="L9" s="10"/>
@@ -2302,15 +2306,15 @@
       <c r="T9" s="10"/>
       <c r="U9" s="11" t="n">
         <f aca="false">SUM(C9:H9)</f>
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="V9" s="11" t="n">
         <f aca="false">SUM(I9:T9)</f>
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="W9" s="12" t="n">
         <f aca="false">SUM(C9:T9)</f>
-        <v>0</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2318,7 +2322,7 @@
         <v>31</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
@@ -2356,14 +2360,16 @@
         <v>32</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
+      <c r="H11" s="10" t="n">
+        <v>16500</v>
+      </c>
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
@@ -2378,7 +2384,7 @@
       <c r="T11" s="10"/>
       <c r="U11" s="11" t="n">
         <f aca="false">SUM(C11:H11)</f>
-        <v>0</v>
+        <v>16500</v>
       </c>
       <c r="V11" s="11" t="n">
         <f aca="false">SUM(I11:T11)</f>
@@ -2386,7 +2392,7 @@
       </c>
       <c r="W11" s="12" t="n">
         <f aca="false">SUM(C11:T11)</f>
-        <v>0</v>
+        <v>16500</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2394,7 +2400,7 @@
         <v>33</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -2430,7 +2436,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13"/>
       <c r="B13" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -2466,7 +2472,7 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -2502,7 +2508,7 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -2538,7 +2544,7 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13"/>
       <c r="B16" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -2574,7 +2580,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
       <c r="B17" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -2608,130 +2614,117 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="16" t="n">
-        <f aca="false">SUM(C9:C17)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="16" t="n">
-        <f aca="false">SUM(D9:D17)</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="16" t="n">
-        <f aca="false">SUM(E9:E17)</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <f aca="false">SUM(F9:F17)</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="16" t="n">
-        <f aca="false">SUM(G9:G17)</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="16" t="n">
-        <f aca="false">SUM(H9:H17)</f>
-        <v>0</v>
-      </c>
-      <c r="I18" s="16" t="n">
-        <f aca="false">SUM(I9:I17)</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="16" t="n">
-        <f aca="false">SUM(J9:J17)</f>
-        <v>0</v>
-      </c>
-      <c r="K18" s="16" t="n">
-        <f aca="false">SUM(K9:K17)</f>
-        <v>0</v>
-      </c>
-      <c r="L18" s="16" t="n">
-        <f aca="false">SUM(L9:L17)</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="16" t="n">
-        <f aca="false">SUM(M9:M17)</f>
-        <v>0</v>
-      </c>
-      <c r="N18" s="16" t="n">
-        <f aca="false">SUM(N9:N17)</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="16" t="n">
-        <f aca="false">SUM(O9:O17)</f>
-        <v>0</v>
-      </c>
-      <c r="P18" s="16" t="n">
-        <f aca="false">SUM(P9:P17)</f>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="16" t="n">
-        <f aca="false">SUM(Q9:Q17)</f>
-        <v>0</v>
-      </c>
-      <c r="R18" s="16" t="n">
-        <f aca="false">SUM(R9:R17)</f>
-        <v>0</v>
-      </c>
-      <c r="S18" s="16" t="n">
-        <f aca="false">SUM(S9:S17)</f>
-        <v>0</v>
-      </c>
-      <c r="T18" s="16" t="n">
-        <f aca="false">SUM(T9:T17)</f>
-        <v>0</v>
-      </c>
-      <c r="U18" s="16" t="n">
-        <f aca="false">SUM(U9:U17)</f>
-        <v>0</v>
-      </c>
-      <c r="V18" s="16" t="n">
-        <f aca="false">SUM(V9:V17)</f>
-        <v>0</v>
-      </c>
-      <c r="W18" s="16" t="n">
-        <f aca="false">SUM(W9:W17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="7"/>
-      <c r="V20" s="7"/>
-      <c r="W20" s="7"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="11" t="n">
+        <f aca="false">SUM(C18:H18)</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="11" t="n">
+        <f aca="false">SUM(I18:T18)</f>
+        <v>0</v>
+      </c>
+      <c r="W18" s="12" t="n">
+        <f aca="false">SUM(C18:T18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+      <c r="B19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="11" t="n">
+        <f aca="false">SUM(C19:H19)</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="11" t="n">
+        <f aca="false">SUM(I19:T19)</f>
+        <v>0</v>
+      </c>
+      <c r="W19" s="12" t="n">
+        <f aca="false">SUM(C19:T19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="B20" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="11" t="n">
+        <f aca="false">SUM(C20:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="V20" s="11" t="n">
+        <f aca="false">SUM(I20:T20)</f>
+        <v>0</v>
+      </c>
+      <c r="W20" s="12" t="n">
+        <f aca="false">SUM(C20:T20)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="A21" s="13"/>
       <c r="B21" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -2765,11 +2758,9 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
-        <v>38</v>
-      </c>
+      <c r="A22" s="13"/>
       <c r="B22" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -2803,11 +2794,9 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>39</v>
-      </c>
+      <c r="A23" s="13"/>
       <c r="B23" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
@@ -2841,11 +2830,9 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>40</v>
-      </c>
+      <c r="A24" s="13"/>
       <c r="B24" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -2879,11 +2866,9 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
-        <v>41</v>
-      </c>
+      <c r="A25" s="13"/>
       <c r="B25" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -2917,11 +2902,9 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
-        <v>42</v>
-      </c>
+      <c r="A26" s="13"/>
       <c r="B26" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -2955,11 +2938,9 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>43</v>
-      </c>
+      <c r="A27" s="13"/>
       <c r="B27" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -2993,11 +2974,9 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>44</v>
-      </c>
+      <c r="A28" s="13"/>
       <c r="B28" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -3031,11 +3010,9 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
-        <v>45</v>
-      </c>
+      <c r="A29" s="13"/>
       <c r="B29" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
@@ -3069,11 +3046,9 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>46</v>
-      </c>
+      <c r="A30" s="13"/>
       <c r="B30" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
@@ -3107,11 +3082,9 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="s">
-        <v>47</v>
-      </c>
+      <c r="A31" s="13"/>
       <c r="B31" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
@@ -3147,7 +3120,7 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13"/>
       <c r="B32" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
@@ -3183,7 +3156,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13"/>
       <c r="B33" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
@@ -3219,7 +3192,7 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13"/>
       <c r="B34" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
@@ -3255,7 +3228,7 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13"/>
       <c r="B35" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -3291,7 +3264,7 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13"/>
       <c r="B36" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
@@ -3327,7 +3300,7 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13"/>
       <c r="B37" s="9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
@@ -3361,568 +3334,1745 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13"/>
-      <c r="B38" s="9" t="s">
+      <c r="A38" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="16" t="n">
+        <f aca="false">SUM(C8:C37)</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="16" t="n">
+        <f aca="false">SUM(D8:D37)</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="16" t="n">
+        <f aca="false">SUM(E8:E37)</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <f aca="false">SUM(F8:F37)</f>
+        <v>20000</v>
+      </c>
+      <c r="G38" s="16" t="n">
+        <f aca="false">SUM(G8:G37)</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="16" t="n">
+        <f aca="false">SUM(H8:H37)</f>
+        <v>16500</v>
+      </c>
+      <c r="I38" s="16" t="n">
+        <f aca="false">SUM(I8:I37)</f>
+        <v>20000</v>
+      </c>
+      <c r="J38" s="16" t="n">
+        <f aca="false">SUM(J8:J37)</f>
+        <v>0</v>
+      </c>
+      <c r="K38" s="16" t="n">
+        <f aca="false">SUM(K8:K37)</f>
+        <v>0</v>
+      </c>
+      <c r="L38" s="16" t="n">
+        <f aca="false">SUM(L8:L37)</f>
+        <v>0</v>
+      </c>
+      <c r="M38" s="16" t="n">
+        <f aca="false">SUM(M8:M37)</f>
+        <v>0</v>
+      </c>
+      <c r="N38" s="16" t="n">
+        <f aca="false">SUM(N8:N37)</f>
+        <v>0</v>
+      </c>
+      <c r="O38" s="16" t="n">
+        <f aca="false">SUM(O8:O37)</f>
+        <v>0</v>
+      </c>
+      <c r="P38" s="16" t="n">
+        <f aca="false">SUM(P8:P37)</f>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="16" t="n">
+        <f aca="false">SUM(Q8:Q37)</f>
+        <v>0</v>
+      </c>
+      <c r="R38" s="16" t="n">
+        <f aca="false">SUM(R8:R37)</f>
+        <v>0</v>
+      </c>
+      <c r="S38" s="16" t="n">
+        <f aca="false">SUM(S8:S37)</f>
+        <v>0</v>
+      </c>
+      <c r="T38" s="16" t="n">
+        <f aca="false">SUM(T8:T37)</f>
+        <v>0</v>
+      </c>
+      <c r="U38" s="16" t="n">
+        <f aca="false">SUM(U8:U37)</f>
+        <v>36500</v>
+      </c>
+      <c r="V38" s="16" t="n">
+        <f aca="false">SUM(V8:V37)</f>
+        <v>20000</v>
+      </c>
+      <c r="W38" s="16" t="n">
+        <f aca="false">SUM(W8:W37)</f>
+        <v>56500</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="7"/>
+      <c r="O40" s="7"/>
+      <c r="P40" s="7"/>
+      <c r="Q40" s="7"/>
+      <c r="R40" s="7"/>
+      <c r="S40" s="7"/>
+      <c r="T40" s="7"/>
+      <c r="U40" s="7"/>
+      <c r="V40" s="7"/>
+      <c r="W40" s="7"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+      <c r="N41" s="10"/>
+      <c r="O41" s="10"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="10"/>
+      <c r="S41" s="10"/>
+      <c r="T41" s="10"/>
+      <c r="U41" s="11" t="n">
+        <f aca="false">SUM(C41:H41)</f>
+        <v>0</v>
+      </c>
+      <c r="V41" s="11" t="n">
+        <f aca="false">SUM(I41:T41)</f>
+        <v>0</v>
+      </c>
+      <c r="W41" s="12" t="n">
+        <f aca="false">SUM(C41:T41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
+      <c r="O42" s="10"/>
+      <c r="P42" s="10"/>
+      <c r="Q42" s="10"/>
+      <c r="R42" s="10"/>
+      <c r="S42" s="10"/>
+      <c r="T42" s="10"/>
+      <c r="U42" s="11" t="n">
+        <f aca="false">SUM(C42:H42)</f>
+        <v>15000</v>
+      </c>
+      <c r="V42" s="11" t="n">
+        <f aca="false">SUM(I42:T42)</f>
+        <v>15000</v>
+      </c>
+      <c r="W42" s="12" t="n">
+        <f aca="false">SUM(C42:T42)</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="10"/>
+      <c r="U43" s="11" t="n">
+        <f aca="false">SUM(C43:H43)</f>
+        <v>0</v>
+      </c>
+      <c r="V43" s="11" t="n">
+        <f aca="false">SUM(I43:T43)</f>
+        <v>0</v>
+      </c>
+      <c r="W43" s="12" t="n">
+        <f aca="false">SUM(C43:T43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10"/>
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="10"/>
+      <c r="R44" s="10"/>
+      <c r="S44" s="10"/>
+      <c r="T44" s="10"/>
+      <c r="U44" s="11" t="n">
+        <f aca="false">SUM(C44:H44)</f>
+        <v>0</v>
+      </c>
+      <c r="V44" s="11" t="n">
+        <f aca="false">SUM(I44:T44)</f>
+        <v>0</v>
+      </c>
+      <c r="W44" s="12" t="n">
+        <f aca="false">SUM(C44:T44)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="10"/>
+      <c r="M45" s="10"/>
+      <c r="N45" s="10"/>
+      <c r="O45" s="10"/>
+      <c r="P45" s="10"/>
+      <c r="Q45" s="10"/>
+      <c r="R45" s="10"/>
+      <c r="S45" s="10"/>
+      <c r="T45" s="10"/>
+      <c r="U45" s="11" t="n">
+        <f aca="false">SUM(C45:H45)</f>
+        <v>0</v>
+      </c>
+      <c r="V45" s="11" t="n">
+        <f aca="false">SUM(I45:T45)</f>
+        <v>0</v>
+      </c>
+      <c r="W45" s="12" t="n">
+        <f aca="false">SUM(C45:T45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13"/>
+      <c r="B46" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="10"/>
+      <c r="Q46" s="10"/>
+      <c r="R46" s="10"/>
+      <c r="S46" s="10"/>
+      <c r="T46" s="10"/>
+      <c r="U46" s="11" t="n">
+        <f aca="false">SUM(C46:H46)</f>
+        <v>0</v>
+      </c>
+      <c r="V46" s="11" t="n">
+        <f aca="false">SUM(I46:T46)</f>
+        <v>0</v>
+      </c>
+      <c r="W46" s="12" t="n">
+        <f aca="false">SUM(C46:T46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13"/>
+      <c r="B47" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10"/>
+      <c r="L47" s="10"/>
+      <c r="M47" s="10"/>
+      <c r="N47" s="10"/>
+      <c r="O47" s="10"/>
+      <c r="P47" s="10"/>
+      <c r="Q47" s="10"/>
+      <c r="R47" s="10"/>
+      <c r="S47" s="10"/>
+      <c r="T47" s="10"/>
+      <c r="U47" s="11" t="n">
+        <f aca="false">SUM(C47:H47)</f>
+        <v>0</v>
+      </c>
+      <c r="V47" s="11" t="n">
+        <f aca="false">SUM(I47:T47)</f>
+        <v>0</v>
+      </c>
+      <c r="W47" s="12" t="n">
+        <f aca="false">SUM(C47:T47)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13"/>
+      <c r="B48" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="10"/>
+      <c r="L48" s="10"/>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="10"/>
+      <c r="Q48" s="10"/>
+      <c r="R48" s="10"/>
+      <c r="S48" s="10"/>
+      <c r="T48" s="10"/>
+      <c r="U48" s="11" t="n">
+        <f aca="false">SUM(C48:H48)</f>
+        <v>0</v>
+      </c>
+      <c r="V48" s="11" t="n">
+        <f aca="false">SUM(I48:T48)</f>
+        <v>0</v>
+      </c>
+      <c r="W48" s="12" t="n">
+        <f aca="false">SUM(C48:T48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13"/>
+      <c r="B49" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+      <c r="O49" s="10"/>
+      <c r="P49" s="10"/>
+      <c r="Q49" s="10"/>
+      <c r="R49" s="10"/>
+      <c r="S49" s="10"/>
+      <c r="T49" s="10"/>
+      <c r="U49" s="11" t="n">
+        <f aca="false">SUM(C49:H49)</f>
+        <v>0</v>
+      </c>
+      <c r="V49" s="11" t="n">
+        <f aca="false">SUM(I49:T49)</f>
+        <v>0</v>
+      </c>
+      <c r="W49" s="12" t="n">
+        <f aca="false">SUM(C49:T49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13"/>
+      <c r="B50" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="10"/>
+      <c r="K50" s="10"/>
+      <c r="L50" s="10"/>
+      <c r="M50" s="10"/>
+      <c r="N50" s="10"/>
+      <c r="O50" s="10"/>
+      <c r="P50" s="10"/>
+      <c r="Q50" s="10"/>
+      <c r="R50" s="10"/>
+      <c r="S50" s="10"/>
+      <c r="T50" s="10"/>
+      <c r="U50" s="11" t="n">
+        <f aca="false">SUM(C50:H50)</f>
+        <v>0</v>
+      </c>
+      <c r="V50" s="11" t="n">
+        <f aca="false">SUM(I50:T50)</f>
+        <v>0</v>
+      </c>
+      <c r="W50" s="12" t="n">
+        <f aca="false">SUM(C50:T50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="13"/>
+      <c r="B51" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
+      <c r="L51" s="10"/>
+      <c r="M51" s="10"/>
+      <c r="N51" s="10"/>
+      <c r="O51" s="10"/>
+      <c r="P51" s="10"/>
+      <c r="Q51" s="10"/>
+      <c r="R51" s="10"/>
+      <c r="S51" s="10"/>
+      <c r="T51" s="10"/>
+      <c r="U51" s="11" t="n">
+        <f aca="false">SUM(C51:H51)</f>
+        <v>0</v>
+      </c>
+      <c r="V51" s="11" t="n">
+        <f aca="false">SUM(I51:T51)</f>
+        <v>0</v>
+      </c>
+      <c r="W51" s="12" t="n">
+        <f aca="false">SUM(C51:T51)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="13"/>
+      <c r="B52" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="10"/>
+      <c r="H52" s="10"/>
+      <c r="I52" s="10"/>
+      <c r="J52" s="10"/>
+      <c r="K52" s="10"/>
+      <c r="L52" s="10"/>
+      <c r="M52" s="10"/>
+      <c r="N52" s="10"/>
+      <c r="O52" s="10"/>
+      <c r="P52" s="10"/>
+      <c r="Q52" s="10"/>
+      <c r="R52" s="10"/>
+      <c r="S52" s="10"/>
+      <c r="T52" s="10"/>
+      <c r="U52" s="11" t="n">
+        <f aca="false">SUM(C52:H52)</f>
+        <v>0</v>
+      </c>
+      <c r="V52" s="11" t="n">
+        <f aca="false">SUM(I52:T52)</f>
+        <v>0</v>
+      </c>
+      <c r="W52" s="12" t="n">
+        <f aca="false">SUM(C52:T52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13"/>
+      <c r="B53" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="10"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="10"/>
+      <c r="I53" s="10"/>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10"/>
+      <c r="L53" s="10"/>
+      <c r="M53" s="10"/>
+      <c r="N53" s="10"/>
+      <c r="O53" s="10"/>
+      <c r="P53" s="10"/>
+      <c r="Q53" s="10"/>
+      <c r="R53" s="10"/>
+      <c r="S53" s="10"/>
+      <c r="T53" s="10"/>
+      <c r="U53" s="11" t="n">
+        <f aca="false">SUM(C53:H53)</f>
+        <v>0</v>
+      </c>
+      <c r="V53" s="11" t="n">
+        <f aca="false">SUM(I53:T53)</f>
+        <v>0</v>
+      </c>
+      <c r="W53" s="12" t="n">
+        <f aca="false">SUM(C53:T53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="13"/>
+      <c r="B54" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="10"/>
+      <c r="J54" s="10"/>
+      <c r="K54" s="10"/>
+      <c r="L54" s="10"/>
+      <c r="M54" s="10"/>
+      <c r="N54" s="10"/>
+      <c r="O54" s="10"/>
+      <c r="P54" s="10"/>
+      <c r="Q54" s="10"/>
+      <c r="R54" s="10"/>
+      <c r="S54" s="10"/>
+      <c r="T54" s="10"/>
+      <c r="U54" s="11" t="n">
+        <f aca="false">SUM(C54:H54)</f>
+        <v>0</v>
+      </c>
+      <c r="V54" s="11" t="n">
+        <f aca="false">SUM(I54:T54)</f>
+        <v>0</v>
+      </c>
+      <c r="W54" s="12" t="n">
+        <f aca="false">SUM(C54:T54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="13"/>
+      <c r="B55" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10"/>
+      <c r="L55" s="10"/>
+      <c r="M55" s="10"/>
+      <c r="N55" s="10"/>
+      <c r="O55" s="10"/>
+      <c r="P55" s="10"/>
+      <c r="Q55" s="10"/>
+      <c r="R55" s="10"/>
+      <c r="S55" s="10"/>
+      <c r="T55" s="10"/>
+      <c r="U55" s="11" t="n">
+        <f aca="false">SUM(C55:H55)</f>
+        <v>0</v>
+      </c>
+      <c r="V55" s="11" t="n">
+        <f aca="false">SUM(I55:T55)</f>
+        <v>0</v>
+      </c>
+      <c r="W55" s="12" t="n">
+        <f aca="false">SUM(C55:T55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="13"/>
+      <c r="B56" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="10"/>
+      <c r="K56" s="10"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="10"/>
+      <c r="N56" s="10"/>
+      <c r="O56" s="10"/>
+      <c r="P56" s="10"/>
+      <c r="Q56" s="10"/>
+      <c r="R56" s="10"/>
+      <c r="S56" s="10"/>
+      <c r="T56" s="10"/>
+      <c r="U56" s="11" t="n">
+        <f aca="false">SUM(C56:H56)</f>
+        <v>0</v>
+      </c>
+      <c r="V56" s="11" t="n">
+        <f aca="false">SUM(I56:T56)</f>
+        <v>0</v>
+      </c>
+      <c r="W56" s="12" t="n">
+        <f aca="false">SUM(C56:T56)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="13"/>
+      <c r="B57" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C57" s="10"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10"/>
+      <c r="J57" s="10"/>
+      <c r="K57" s="10"/>
+      <c r="L57" s="10"/>
+      <c r="M57" s="10"/>
+      <c r="N57" s="10"/>
+      <c r="O57" s="10"/>
+      <c r="P57" s="10"/>
+      <c r="Q57" s="10"/>
+      <c r="R57" s="10"/>
+      <c r="S57" s="10"/>
+      <c r="T57" s="10"/>
+      <c r="U57" s="11" t="n">
+        <f aca="false">SUM(C57:H57)</f>
+        <v>0</v>
+      </c>
+      <c r="V57" s="11" t="n">
+        <f aca="false">SUM(I57:T57)</f>
+        <v>0</v>
+      </c>
+      <c r="W57" s="12" t="n">
+        <f aca="false">SUM(C57:T57)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="13"/>
+      <c r="B58" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10"/>
+      <c r="J58" s="10"/>
+      <c r="K58" s="10"/>
+      <c r="L58" s="10"/>
+      <c r="M58" s="10"/>
+      <c r="N58" s="10"/>
+      <c r="O58" s="10"/>
+      <c r="P58" s="10"/>
+      <c r="Q58" s="10"/>
+      <c r="R58" s="10"/>
+      <c r="S58" s="10"/>
+      <c r="T58" s="10"/>
+      <c r="U58" s="11" t="n">
+        <f aca="false">SUM(C58:H58)</f>
+        <v>0</v>
+      </c>
+      <c r="V58" s="11" t="n">
+        <f aca="false">SUM(I58:T58)</f>
+        <v>0</v>
+      </c>
+      <c r="W58" s="12" t="n">
+        <f aca="false">SUM(C58:T58)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="13"/>
+      <c r="B59" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="10"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10"/>
+      <c r="I59" s="10"/>
+      <c r="J59" s="10"/>
+      <c r="K59" s="10"/>
+      <c r="L59" s="10"/>
+      <c r="M59" s="10"/>
+      <c r="N59" s="10"/>
+      <c r="O59" s="10"/>
+      <c r="P59" s="10"/>
+      <c r="Q59" s="10"/>
+      <c r="R59" s="10"/>
+      <c r="S59" s="10"/>
+      <c r="T59" s="10"/>
+      <c r="U59" s="11" t="n">
+        <f aca="false">SUM(C59:H59)</f>
+        <v>0</v>
+      </c>
+      <c r="V59" s="11" t="n">
+        <f aca="false">SUM(I59:T59)</f>
+        <v>0</v>
+      </c>
+      <c r="W59" s="12" t="n">
+        <f aca="false">SUM(C59:T59)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="13"/>
+      <c r="B60" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10"/>
+      <c r="I60" s="10"/>
+      <c r="J60" s="10"/>
+      <c r="K60" s="10"/>
+      <c r="L60" s="10"/>
+      <c r="M60" s="10"/>
+      <c r="N60" s="10"/>
+      <c r="O60" s="10"/>
+      <c r="P60" s="10"/>
+      <c r="Q60" s="10"/>
+      <c r="R60" s="10"/>
+      <c r="S60" s="10"/>
+      <c r="T60" s="10"/>
+      <c r="U60" s="11" t="n">
+        <f aca="false">SUM(C60:H60)</f>
+        <v>0</v>
+      </c>
+      <c r="V60" s="11" t="n">
+        <f aca="false">SUM(I60:T60)</f>
+        <v>0</v>
+      </c>
+      <c r="W60" s="12" t="n">
+        <f aca="false">SUM(C60:T60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="13"/>
+      <c r="B61" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="10"/>
+      <c r="J61" s="10"/>
+      <c r="K61" s="10"/>
+      <c r="L61" s="10"/>
+      <c r="M61" s="10"/>
+      <c r="N61" s="10"/>
+      <c r="O61" s="10"/>
+      <c r="P61" s="10"/>
+      <c r="Q61" s="10"/>
+      <c r="R61" s="10"/>
+      <c r="S61" s="10"/>
+      <c r="T61" s="10"/>
+      <c r="U61" s="11" t="n">
+        <f aca="false">SUM(C61:H61)</f>
+        <v>0</v>
+      </c>
+      <c r="V61" s="11" t="n">
+        <f aca="false">SUM(I61:T61)</f>
+        <v>0</v>
+      </c>
+      <c r="W61" s="12" t="n">
+        <f aca="false">SUM(C61:T61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13"/>
+      <c r="B62" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C62" s="10"/>
+      <c r="D62" s="10"/>
+      <c r="E62" s="10"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="10"/>
+      <c r="H62" s="10"/>
+      <c r="I62" s="10"/>
+      <c r="J62" s="10"/>
+      <c r="K62" s="10"/>
+      <c r="L62" s="10"/>
+      <c r="M62" s="10"/>
+      <c r="N62" s="10"/>
+      <c r="O62" s="10"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="10"/>
+      <c r="R62" s="10"/>
+      <c r="S62" s="10"/>
+      <c r="T62" s="10"/>
+      <c r="U62" s="11" t="n">
+        <f aca="false">SUM(C62:H62)</f>
+        <v>0</v>
+      </c>
+      <c r="V62" s="11" t="n">
+        <f aca="false">SUM(I62:T62)</f>
+        <v>0</v>
+      </c>
+      <c r="W62" s="12" t="n">
+        <f aca="false">SUM(C62:T62)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13"/>
+      <c r="B63" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+      <c r="I63" s="10"/>
+      <c r="J63" s="10"/>
+      <c r="K63" s="10"/>
+      <c r="L63" s="10"/>
+      <c r="M63" s="10"/>
+      <c r="N63" s="10"/>
+      <c r="O63" s="10"/>
+      <c r="P63" s="10"/>
+      <c r="Q63" s="10"/>
+      <c r="R63" s="10"/>
+      <c r="S63" s="10"/>
+      <c r="T63" s="10"/>
+      <c r="U63" s="11" t="n">
+        <f aca="false">SUM(C63:H63)</f>
+        <v>0</v>
+      </c>
+      <c r="V63" s="11" t="n">
+        <f aca="false">SUM(I63:T63)</f>
+        <v>0</v>
+      </c>
+      <c r="W63" s="12" t="n">
+        <f aca="false">SUM(C63:T63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="13"/>
+      <c r="B64" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C64" s="10"/>
+      <c r="D64" s="10"/>
+      <c r="E64" s="10"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+      <c r="I64" s="10"/>
+      <c r="J64" s="10"/>
+      <c r="K64" s="10"/>
+      <c r="L64" s="10"/>
+      <c r="M64" s="10"/>
+      <c r="N64" s="10"/>
+      <c r="O64" s="10"/>
+      <c r="P64" s="10"/>
+      <c r="Q64" s="10"/>
+      <c r="R64" s="10"/>
+      <c r="S64" s="10"/>
+      <c r="T64" s="10"/>
+      <c r="U64" s="11" t="n">
+        <f aca="false">SUM(C64:H64)</f>
+        <v>0</v>
+      </c>
+      <c r="V64" s="11" t="n">
+        <f aca="false">SUM(I64:T64)</f>
+        <v>0</v>
+      </c>
+      <c r="W64" s="12" t="n">
+        <f aca="false">SUM(C64:T64)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="13"/>
+      <c r="B65" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C65" s="10"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10"/>
+      <c r="F65" s="10"/>
+      <c r="G65" s="10"/>
+      <c r="H65" s="10"/>
+      <c r="I65" s="10"/>
+      <c r="J65" s="10"/>
+      <c r="K65" s="10"/>
+      <c r="L65" s="10"/>
+      <c r="M65" s="10"/>
+      <c r="N65" s="10"/>
+      <c r="O65" s="10"/>
+      <c r="P65" s="10"/>
+      <c r="Q65" s="10"/>
+      <c r="R65" s="10"/>
+      <c r="S65" s="10"/>
+      <c r="T65" s="10"/>
+      <c r="U65" s="11" t="n">
+        <f aca="false">SUM(C65:H65)</f>
+        <v>0</v>
+      </c>
+      <c r="V65" s="11" t="n">
+        <f aca="false">SUM(I65:T65)</f>
+        <v>0</v>
+      </c>
+      <c r="W65" s="12" t="n">
+        <f aca="false">SUM(C65:T65)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="13"/>
+      <c r="B66" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="10"/>
+      <c r="I66" s="10"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="10"/>
+      <c r="L66" s="10"/>
+      <c r="M66" s="10"/>
+      <c r="N66" s="10"/>
+      <c r="O66" s="10"/>
+      <c r="P66" s="10"/>
+      <c r="Q66" s="10"/>
+      <c r="R66" s="10"/>
+      <c r="S66" s="10"/>
+      <c r="T66" s="10"/>
+      <c r="U66" s="11" t="n">
+        <f aca="false">SUM(C66:H66)</f>
+        <v>0</v>
+      </c>
+      <c r="V66" s="11" t="n">
+        <f aca="false">SUM(I66:T66)</f>
+        <v>0</v>
+      </c>
+      <c r="W66" s="12" t="n">
+        <f aca="false">SUM(C66:T66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13"/>
+      <c r="B67" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C67" s="10"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="10"/>
+      <c r="I67" s="10"/>
+      <c r="J67" s="10"/>
+      <c r="K67" s="10"/>
+      <c r="L67" s="10"/>
+      <c r="M67" s="10"/>
+      <c r="N67" s="10"/>
+      <c r="O67" s="10"/>
+      <c r="P67" s="10"/>
+      <c r="Q67" s="10"/>
+      <c r="R67" s="10"/>
+      <c r="S67" s="10"/>
+      <c r="T67" s="10"/>
+      <c r="U67" s="11" t="n">
+        <f aca="false">SUM(C67:H67)</f>
+        <v>0</v>
+      </c>
+      <c r="V67" s="11" t="n">
+        <f aca="false">SUM(I67:T67)</f>
+        <v>0</v>
+      </c>
+      <c r="W67" s="12" t="n">
+        <f aca="false">SUM(C67:T67)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13"/>
+      <c r="B68" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68" s="10"/>
+      <c r="D68" s="10"/>
+      <c r="E68" s="10"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+      <c r="I68" s="10"/>
+      <c r="J68" s="10"/>
+      <c r="K68" s="10"/>
+      <c r="L68" s="10"/>
+      <c r="M68" s="10"/>
+      <c r="N68" s="10"/>
+      <c r="O68" s="10"/>
+      <c r="P68" s="10"/>
+      <c r="Q68" s="10"/>
+      <c r="R68" s="10"/>
+      <c r="S68" s="10"/>
+      <c r="T68" s="10"/>
+      <c r="U68" s="11" t="n">
+        <f aca="false">SUM(C68:H68)</f>
+        <v>0</v>
+      </c>
+      <c r="V68" s="11" t="n">
+        <f aca="false">SUM(I68:T68)</f>
+        <v>0</v>
+      </c>
+      <c r="W68" s="12" t="n">
+        <f aca="false">SUM(C68:T68)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13"/>
+      <c r="B69" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="10"/>
+      <c r="G69" s="10"/>
+      <c r="H69" s="10"/>
+      <c r="I69" s="10"/>
+      <c r="J69" s="10"/>
+      <c r="K69" s="10"/>
+      <c r="L69" s="10"/>
+      <c r="M69" s="10"/>
+      <c r="N69" s="10"/>
+      <c r="O69" s="10"/>
+      <c r="P69" s="10"/>
+      <c r="Q69" s="10"/>
+      <c r="R69" s="10"/>
+      <c r="S69" s="10"/>
+      <c r="T69" s="10"/>
+      <c r="U69" s="11" t="n">
+        <f aca="false">SUM(C69:H69)</f>
+        <v>0</v>
+      </c>
+      <c r="V69" s="11" t="n">
+        <f aca="false">SUM(I69:T69)</f>
+        <v>0</v>
+      </c>
+      <c r="W69" s="12" t="n">
+        <f aca="false">SUM(C69:T69)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13"/>
+      <c r="B70" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C70" s="10"/>
+      <c r="D70" s="10"/>
+      <c r="E70" s="10"/>
+      <c r="F70" s="10"/>
+      <c r="G70" s="10"/>
+      <c r="H70" s="10"/>
+      <c r="I70" s="10"/>
+      <c r="J70" s="10"/>
+      <c r="K70" s="10"/>
+      <c r="L70" s="10"/>
+      <c r="M70" s="10"/>
+      <c r="N70" s="10"/>
+      <c r="O70" s="10"/>
+      <c r="P70" s="10"/>
+      <c r="Q70" s="10"/>
+      <c r="R70" s="10"/>
+      <c r="S70" s="10"/>
+      <c r="T70" s="10"/>
+      <c r="U70" s="11" t="n">
+        <f aca="false">SUM(C70:H70)</f>
+        <v>0</v>
+      </c>
+      <c r="V70" s="11" t="n">
+        <f aca="false">SUM(I70:T70)</f>
+        <v>0</v>
+      </c>
+      <c r="W70" s="12" t="n">
+        <f aca="false">SUM(C70:T70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="10"/>
-      <c r="S38" s="10"/>
-      <c r="T38" s="10"/>
-      <c r="U38" s="11" t="n">
-        <f aca="false">SUM(C38:H38)</f>
-        <v>0</v>
-      </c>
-      <c r="V38" s="11" t="n">
-        <f aca="false">SUM(I38:T38)</f>
-        <v>0</v>
-      </c>
-      <c r="W38" s="12" t="n">
-        <f aca="false">SUM(C38:T38)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="15" t="s">
+      <c r="B71" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C71" s="16" t="n">
+        <f aca="false">SUM(C41:C70)</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="16" t="n">
+        <f aca="false">SUM(D41:D70)</f>
+        <v>0</v>
+      </c>
+      <c r="E71" s="16" t="n">
+        <f aca="false">SUM(E41:E70)</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="16" t="n">
+        <f aca="false">SUM(F41:F70)</f>
+        <v>15000</v>
+      </c>
+      <c r="G71" s="16" t="n">
+        <f aca="false">SUM(G41:G70)</f>
+        <v>0</v>
+      </c>
+      <c r="H71" s="16" t="n">
+        <f aca="false">SUM(H41:H70)</f>
+        <v>0</v>
+      </c>
+      <c r="I71" s="16" t="n">
+        <f aca="false">SUM(I41:I70)</f>
+        <v>15000</v>
+      </c>
+      <c r="J71" s="16" t="n">
+        <f aca="false">SUM(J41:J70)</f>
+        <v>0</v>
+      </c>
+      <c r="K71" s="16" t="n">
+        <f aca="false">SUM(K41:K70)</f>
+        <v>0</v>
+      </c>
+      <c r="L71" s="16" t="n">
+        <f aca="false">SUM(L41:L70)</f>
+        <v>0</v>
+      </c>
+      <c r="M71" s="16" t="n">
+        <f aca="false">SUM(M41:M70)</f>
+        <v>0</v>
+      </c>
+      <c r="N71" s="16" t="n">
+        <f aca="false">SUM(N41:N70)</f>
+        <v>0</v>
+      </c>
+      <c r="O71" s="16" t="n">
+        <f aca="false">SUM(O41:O70)</f>
+        <v>0</v>
+      </c>
+      <c r="P71" s="16" t="n">
+        <f aca="false">SUM(P41:P70)</f>
+        <v>0</v>
+      </c>
+      <c r="Q71" s="16" t="n">
+        <f aca="false">SUM(Q41:Q70)</f>
+        <v>0</v>
+      </c>
+      <c r="R71" s="16" t="n">
+        <f aca="false">SUM(R41:R70)</f>
+        <v>0</v>
+      </c>
+      <c r="S71" s="16" t="n">
+        <f aca="false">SUM(S41:S70)</f>
+        <v>0</v>
+      </c>
+      <c r="T71" s="16" t="n">
+        <f aca="false">SUM(T41:T70)</f>
+        <v>0</v>
+      </c>
+      <c r="U71" s="16" t="n">
+        <f aca="false">SUM(U41:U70)</f>
+        <v>15000</v>
+      </c>
+      <c r="V71" s="16" t="n">
+        <f aca="false">SUM(V41:V70)</f>
+        <v>15000</v>
+      </c>
+      <c r="W71" s="16" t="n">
+        <f aca="false">SUM(W41:W70)</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="7"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
+      <c r="N73" s="7"/>
+      <c r="O73" s="7"/>
+      <c r="P73" s="7"/>
+      <c r="Q73" s="7"/>
+      <c r="R73" s="7"/>
+      <c r="S73" s="7"/>
+      <c r="T73" s="7"/>
+      <c r="U73" s="7"/>
+      <c r="V73" s="7"/>
+      <c r="W73" s="7"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C74" s="11" t="n">
+        <f aca="false">C38</f>
+        <v>0</v>
+      </c>
+      <c r="D74" s="11" t="n">
+        <f aca="false">D38</f>
+        <v>0</v>
+      </c>
+      <c r="E74" s="11" t="n">
+        <f aca="false">E38</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="11" t="n">
+        <f aca="false">F38</f>
+        <v>20000</v>
+      </c>
+      <c r="G74" s="11" t="n">
+        <f aca="false">G38</f>
+        <v>0</v>
+      </c>
+      <c r="H74" s="11" t="n">
+        <f aca="false">H38</f>
+        <v>16500</v>
+      </c>
+      <c r="I74" s="11" t="n">
+        <f aca="false">I38</f>
+        <v>20000</v>
+      </c>
+      <c r="J74" s="11" t="n">
+        <f aca="false">J38</f>
+        <v>0</v>
+      </c>
+      <c r="K74" s="11" t="n">
+        <f aca="false">K38</f>
+        <v>0</v>
+      </c>
+      <c r="L74" s="11" t="n">
+        <f aca="false">L38</f>
+        <v>0</v>
+      </c>
+      <c r="M74" s="11" t="n">
+        <f aca="false">M38</f>
+        <v>0</v>
+      </c>
+      <c r="N74" s="11" t="n">
+        <f aca="false">N38</f>
+        <v>0</v>
+      </c>
+      <c r="O74" s="11" t="n">
+        <f aca="false">O38</f>
+        <v>0</v>
+      </c>
+      <c r="P74" s="11" t="n">
+        <f aca="false">P38</f>
+        <v>0</v>
+      </c>
+      <c r="Q74" s="11" t="n">
+        <f aca="false">Q38</f>
+        <v>0</v>
+      </c>
+      <c r="R74" s="11" t="n">
+        <f aca="false">R38</f>
+        <v>0</v>
+      </c>
+      <c r="S74" s="11" t="n">
+        <f aca="false">S38</f>
+        <v>0</v>
+      </c>
+      <c r="T74" s="11" t="n">
+        <f aca="false">T38</f>
+        <v>0</v>
+      </c>
+      <c r="U74" s="11" t="n">
+        <f aca="false">U38</f>
+        <v>36500</v>
+      </c>
+      <c r="V74" s="11" t="n">
+        <f aca="false">V38</f>
+        <v>20000</v>
+      </c>
+      <c r="W74" s="11" t="n">
+        <f aca="false">W38</f>
+        <v>56500</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="16" t="n">
-        <f aca="false">SUM(C21:C38)</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="16" t="n">
-        <f aca="false">SUM(D21:D38)</f>
-        <v>0</v>
-      </c>
-      <c r="E39" s="16" t="n">
-        <f aca="false">SUM(E21:E38)</f>
-        <v>0</v>
-      </c>
-      <c r="F39" s="16" t="n">
-        <f aca="false">SUM(F21:F38)</f>
-        <v>0</v>
-      </c>
-      <c r="G39" s="16" t="n">
-        <f aca="false">SUM(G21:G38)</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="16" t="n">
-        <f aca="false">SUM(H21:H38)</f>
-        <v>0</v>
-      </c>
-      <c r="I39" s="16" t="n">
-        <f aca="false">SUM(I21:I38)</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="16" t="n">
-        <f aca="false">SUM(J21:J38)</f>
-        <v>0</v>
-      </c>
-      <c r="K39" s="16" t="n">
-        <f aca="false">SUM(K21:K38)</f>
-        <v>0</v>
-      </c>
-      <c r="L39" s="16" t="n">
-        <f aca="false">SUM(L21:L38)</f>
-        <v>0</v>
-      </c>
-      <c r="M39" s="16" t="n">
-        <f aca="false">SUM(M21:M38)</f>
-        <v>0</v>
-      </c>
-      <c r="N39" s="16" t="n">
-        <f aca="false">SUM(N21:N38)</f>
-        <v>0</v>
-      </c>
-      <c r="O39" s="16" t="n">
-        <f aca="false">SUM(O21:O38)</f>
-        <v>0</v>
-      </c>
-      <c r="P39" s="16" t="n">
-        <f aca="false">SUM(P21:P38)</f>
-        <v>0</v>
-      </c>
-      <c r="Q39" s="16" t="n">
-        <f aca="false">SUM(Q21:Q38)</f>
-        <v>0</v>
-      </c>
-      <c r="R39" s="16" t="n">
-        <f aca="false">SUM(R21:R38)</f>
-        <v>0</v>
-      </c>
-      <c r="S39" s="16" t="n">
-        <f aca="false">SUM(S21:S38)</f>
-        <v>0</v>
-      </c>
-      <c r="T39" s="16" t="n">
-        <f aca="false">SUM(T21:T38)</f>
-        <v>0</v>
-      </c>
-      <c r="U39" s="16" t="n">
-        <f aca="false">SUM(U21:U38)</f>
-        <v>0</v>
-      </c>
-      <c r="V39" s="16" t="n">
-        <f aca="false">SUM(V21:V38)</f>
-        <v>0</v>
-      </c>
-      <c r="W39" s="16" t="n">
-        <f aca="false">SUM(W21:W38)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="7"/>
-      <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
-      <c r="L41" s="7"/>
-      <c r="M41" s="7"/>
-      <c r="N41" s="7"/>
-      <c r="O41" s="7"/>
-      <c r="P41" s="7"/>
-      <c r="Q41" s="7"/>
-      <c r="R41" s="7"/>
-      <c r="S41" s="7"/>
-      <c r="T41" s="7"/>
-      <c r="U41" s="7"/>
-      <c r="V41" s="7"/>
-      <c r="W41" s="7"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="B42" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C42" s="11" t="n">
-        <f aca="false">C18</f>
-        <v>0</v>
-      </c>
-      <c r="D42" s="11" t="n">
-        <f aca="false">D18</f>
-        <v>0</v>
-      </c>
-      <c r="E42" s="11" t="n">
-        <f aca="false">E18</f>
-        <v>0</v>
-      </c>
-      <c r="F42" s="11" t="n">
-        <f aca="false">F18</f>
-        <v>0</v>
-      </c>
-      <c r="G42" s="11" t="n">
-        <f aca="false">G18</f>
-        <v>0</v>
-      </c>
-      <c r="H42" s="11" t="n">
-        <f aca="false">H18</f>
-        <v>0</v>
-      </c>
-      <c r="I42" s="11" t="n">
-        <f aca="false">I18</f>
-        <v>0</v>
-      </c>
-      <c r="J42" s="11" t="n">
-        <f aca="false">J18</f>
-        <v>0</v>
-      </c>
-      <c r="K42" s="11" t="n">
-        <f aca="false">K18</f>
-        <v>0</v>
-      </c>
-      <c r="L42" s="11" t="n">
-        <f aca="false">L18</f>
-        <v>0</v>
-      </c>
-      <c r="M42" s="11" t="n">
-        <f aca="false">M18</f>
-        <v>0</v>
-      </c>
-      <c r="N42" s="11" t="n">
-        <f aca="false">N18</f>
-        <v>0</v>
-      </c>
-      <c r="O42" s="11" t="n">
-        <f aca="false">O18</f>
-        <v>0</v>
-      </c>
-      <c r="P42" s="11" t="n">
-        <f aca="false">P18</f>
-        <v>0</v>
-      </c>
-      <c r="Q42" s="11" t="n">
-        <f aca="false">Q18</f>
-        <v>0</v>
-      </c>
-      <c r="R42" s="11" t="n">
-        <f aca="false">R18</f>
-        <v>0</v>
-      </c>
-      <c r="S42" s="11" t="n">
-        <f aca="false">S18</f>
-        <v>0</v>
-      </c>
-      <c r="T42" s="11" t="n">
-        <f aca="false">T18</f>
-        <v>0</v>
-      </c>
-      <c r="U42" s="11" t="n">
-        <f aca="false">U18</f>
-        <v>0</v>
-      </c>
-      <c r="V42" s="11" t="n">
-        <f aca="false">V18</f>
-        <v>0</v>
-      </c>
-      <c r="W42" s="11" t="n">
-        <f aca="false">W18</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" s="11" t="n">
-        <f aca="false">C39</f>
-        <v>0</v>
-      </c>
-      <c r="D43" s="11" t="n">
-        <f aca="false">D39</f>
-        <v>0</v>
-      </c>
-      <c r="E43" s="11" t="n">
-        <f aca="false">E39</f>
-        <v>0</v>
-      </c>
-      <c r="F43" s="11" t="n">
-        <f aca="false">F39</f>
-        <v>0</v>
-      </c>
-      <c r="G43" s="11" t="n">
-        <f aca="false">G39</f>
-        <v>0</v>
-      </c>
-      <c r="H43" s="11" t="n">
-        <f aca="false">H39</f>
-        <v>0</v>
-      </c>
-      <c r="I43" s="11" t="n">
-        <f aca="false">I39</f>
-        <v>0</v>
-      </c>
-      <c r="J43" s="11" t="n">
-        <f aca="false">J39</f>
-        <v>0</v>
-      </c>
-      <c r="K43" s="11" t="n">
-        <f aca="false">K39</f>
-        <v>0</v>
-      </c>
-      <c r="L43" s="11" t="n">
-        <f aca="false">L39</f>
-        <v>0</v>
-      </c>
-      <c r="M43" s="11" t="n">
-        <f aca="false">M39</f>
-        <v>0</v>
-      </c>
-      <c r="N43" s="11" t="n">
-        <f aca="false">N39</f>
-        <v>0</v>
-      </c>
-      <c r="O43" s="11" t="n">
-        <f aca="false">O39</f>
-        <v>0</v>
-      </c>
-      <c r="P43" s="11" t="n">
-        <f aca="false">P39</f>
-        <v>0</v>
-      </c>
-      <c r="Q43" s="11" t="n">
-        <f aca="false">Q39</f>
-        <v>0</v>
-      </c>
-      <c r="R43" s="11" t="n">
-        <f aca="false">R39</f>
-        <v>0</v>
-      </c>
-      <c r="S43" s="11" t="n">
-        <f aca="false">S39</f>
-        <v>0</v>
-      </c>
-      <c r="T43" s="11" t="n">
-        <f aca="false">T39</f>
-        <v>0</v>
-      </c>
-      <c r="U43" s="11" t="n">
-        <f aca="false">U39</f>
-        <v>0</v>
-      </c>
-      <c r="V43" s="11" t="n">
-        <f aca="false">V39</f>
-        <v>0</v>
-      </c>
-      <c r="W43" s="11" t="n">
-        <f aca="false">W39</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="B44" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C44" s="21" t="n">
-        <f aca="false">C42-C43</f>
-        <v>0</v>
-      </c>
-      <c r="D44" s="21" t="n">
-        <f aca="false">D42-D43</f>
-        <v>0</v>
-      </c>
-      <c r="E44" s="21" t="n">
-        <f aca="false">E42-E43</f>
-        <v>0</v>
-      </c>
-      <c r="F44" s="21" t="n">
-        <f aca="false">F42-F43</f>
-        <v>0</v>
-      </c>
-      <c r="G44" s="21" t="n">
-        <f aca="false">G42-G43</f>
-        <v>0</v>
-      </c>
-      <c r="H44" s="21" t="n">
-        <f aca="false">H42-H43</f>
-        <v>0</v>
-      </c>
-      <c r="I44" s="21" t="n">
-        <f aca="false">I42-I43</f>
-        <v>0</v>
-      </c>
-      <c r="J44" s="21" t="n">
-        <f aca="false">J42-J43</f>
-        <v>0</v>
-      </c>
-      <c r="K44" s="21" t="n">
-        <f aca="false">K42-K43</f>
-        <v>0</v>
-      </c>
-      <c r="L44" s="21" t="n">
-        <f aca="false">L42-L43</f>
-        <v>0</v>
-      </c>
-      <c r="M44" s="21" t="n">
-        <f aca="false">M42-M43</f>
-        <v>0</v>
-      </c>
-      <c r="N44" s="21" t="n">
-        <f aca="false">N42-N43</f>
-        <v>0</v>
-      </c>
-      <c r="O44" s="21" t="n">
-        <f aca="false">O42-O43</f>
-        <v>0</v>
-      </c>
-      <c r="P44" s="21" t="n">
-        <f aca="false">P42-P43</f>
-        <v>0</v>
-      </c>
-      <c r="Q44" s="21" t="n">
-        <f aca="false">Q42-Q43</f>
-        <v>0</v>
-      </c>
-      <c r="R44" s="21" t="n">
-        <f aca="false">R42-R43</f>
-        <v>0</v>
-      </c>
-      <c r="S44" s="21" t="n">
-        <f aca="false">S42-S43</f>
-        <v>0</v>
-      </c>
-      <c r="T44" s="21" t="n">
-        <f aca="false">T42-T43</f>
-        <v>0</v>
-      </c>
-      <c r="U44" s="21" t="n">
-        <f aca="false">U42-U43</f>
-        <v>0</v>
-      </c>
-      <c r="V44" s="21" t="n">
-        <f aca="false">V42-V43</f>
-        <v>0</v>
-      </c>
-      <c r="W44" s="21" t="n">
-        <f aca="false">W42-W43</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B45" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C45" s="21" t="n">
-        <f aca="false">C44</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="21" t="n">
-        <f aca="false">C45+D44</f>
-        <v>0</v>
-      </c>
-      <c r="E45" s="21" t="n">
-        <f aca="false">D45+E44</f>
-        <v>0</v>
-      </c>
-      <c r="F45" s="21" t="n">
-        <f aca="false">E45+F44</f>
-        <v>0</v>
-      </c>
-      <c r="G45" s="21" t="n">
-        <f aca="false">F45+G44</f>
-        <v>0</v>
-      </c>
-      <c r="H45" s="21" t="n">
-        <f aca="false">G45+H44</f>
-        <v>0</v>
-      </c>
-      <c r="I45" s="21" t="n">
-        <f aca="false">H45+I44</f>
-        <v>0</v>
-      </c>
-      <c r="J45" s="21" t="n">
-        <f aca="false">I45+J44</f>
-        <v>0</v>
-      </c>
-      <c r="K45" s="21" t="n">
-        <f aca="false">J45+K44</f>
-        <v>0</v>
-      </c>
-      <c r="L45" s="21" t="n">
-        <f aca="false">K45+L44</f>
-        <v>0</v>
-      </c>
-      <c r="M45" s="21" t="n">
-        <f aca="false">L45+M44</f>
-        <v>0</v>
-      </c>
-      <c r="N45" s="21" t="n">
-        <f aca="false">M45+N44</f>
-        <v>0</v>
-      </c>
-      <c r="O45" s="21" t="n">
-        <f aca="false">N45+O44</f>
-        <v>0</v>
-      </c>
-      <c r="P45" s="21" t="n">
-        <f aca="false">O45+P44</f>
-        <v>0</v>
-      </c>
-      <c r="Q45" s="21" t="n">
-        <f aca="false">P45+Q44</f>
-        <v>0</v>
-      </c>
-      <c r="R45" s="21" t="n">
-        <f aca="false">Q45+R44</f>
-        <v>0</v>
-      </c>
-      <c r="S45" s="21" t="n">
-        <f aca="false">R45+S44</f>
-        <v>0</v>
-      </c>
-      <c r="T45" s="21" t="n">
-        <f aca="false">S45+T44</f>
-        <v>0</v>
-      </c>
-      <c r="U45" s="21" t="n">
-        <f aca="false">H45</f>
-        <v>0</v>
-      </c>
-      <c r="V45" s="21" t="n">
-        <f aca="false">T45</f>
-        <v>0</v>
-      </c>
-      <c r="W45" s="21" t="n">
-        <f aca="false">T45</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="23"/>
-      <c r="B49" s="24" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="25"/>
-      <c r="B50" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="26"/>
-      <c r="B51" s="24" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="27" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="27" t="s">
-        <v>58</v>
+      <c r="B75" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C75" s="11" t="n">
+        <f aca="false">C71</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="11" t="n">
+        <f aca="false">D71</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="11" t="n">
+        <f aca="false">E71</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="11" t="n">
+        <f aca="false">F71</f>
+        <v>15000</v>
+      </c>
+      <c r="G75" s="11" t="n">
+        <f aca="false">G71</f>
+        <v>0</v>
+      </c>
+      <c r="H75" s="11" t="n">
+        <f aca="false">H71</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="11" t="n">
+        <f aca="false">I71</f>
+        <v>15000</v>
+      </c>
+      <c r="J75" s="11" t="n">
+        <f aca="false">J71</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="11" t="n">
+        <f aca="false">K71</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="11" t="n">
+        <f aca="false">L71</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="11" t="n">
+        <f aca="false">M71</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="11" t="n">
+        <f aca="false">N71</f>
+        <v>0</v>
+      </c>
+      <c r="O75" s="11" t="n">
+        <f aca="false">O71</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="11" t="n">
+        <f aca="false">P71</f>
+        <v>0</v>
+      </c>
+      <c r="Q75" s="11" t="n">
+        <f aca="false">Q71</f>
+        <v>0</v>
+      </c>
+      <c r="R75" s="11" t="n">
+        <f aca="false">R71</f>
+        <v>0</v>
+      </c>
+      <c r="S75" s="11" t="n">
+        <f aca="false">S71</f>
+        <v>0</v>
+      </c>
+      <c r="T75" s="11" t="n">
+        <f aca="false">T71</f>
+        <v>0</v>
+      </c>
+      <c r="U75" s="11" t="n">
+        <f aca="false">U71</f>
+        <v>15000</v>
+      </c>
+      <c r="V75" s="11" t="n">
+        <f aca="false">V71</f>
+        <v>15000</v>
+      </c>
+      <c r="W75" s="11" t="n">
+        <f aca="false">W71</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C76" s="21" t="n">
+        <f aca="false">C74-C75</f>
+        <v>0</v>
+      </c>
+      <c r="D76" s="21" t="n">
+        <f aca="false">D74-D75</f>
+        <v>0</v>
+      </c>
+      <c r="E76" s="21" t="n">
+        <f aca="false">E74-E75</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="21" t="n">
+        <f aca="false">F74-F75</f>
+        <v>5000</v>
+      </c>
+      <c r="G76" s="21" t="n">
+        <f aca="false">G74-G75</f>
+        <v>0</v>
+      </c>
+      <c r="H76" s="21" t="n">
+        <f aca="false">H74-H75</f>
+        <v>16500</v>
+      </c>
+      <c r="I76" s="21" t="n">
+        <f aca="false">I74-I75</f>
+        <v>5000</v>
+      </c>
+      <c r="J76" s="21" t="n">
+        <f aca="false">J74-J75</f>
+        <v>0</v>
+      </c>
+      <c r="K76" s="21" t="n">
+        <f aca="false">K74-K75</f>
+        <v>0</v>
+      </c>
+      <c r="L76" s="21" t="n">
+        <f aca="false">L74-L75</f>
+        <v>0</v>
+      </c>
+      <c r="M76" s="21" t="n">
+        <f aca="false">M74-M75</f>
+        <v>0</v>
+      </c>
+      <c r="N76" s="21" t="n">
+        <f aca="false">N74-N75</f>
+        <v>0</v>
+      </c>
+      <c r="O76" s="21" t="n">
+        <f aca="false">O74-O75</f>
+        <v>0</v>
+      </c>
+      <c r="P76" s="21" t="n">
+        <f aca="false">P74-P75</f>
+        <v>0</v>
+      </c>
+      <c r="Q76" s="21" t="n">
+        <f aca="false">Q74-Q75</f>
+        <v>0</v>
+      </c>
+      <c r="R76" s="21" t="n">
+        <f aca="false">R74-R75</f>
+        <v>0</v>
+      </c>
+      <c r="S76" s="21" t="n">
+        <f aca="false">S74-S75</f>
+        <v>0</v>
+      </c>
+      <c r="T76" s="21" t="n">
+        <f aca="false">T74-T75</f>
+        <v>0</v>
+      </c>
+      <c r="U76" s="21" t="n">
+        <f aca="false">U74-U75</f>
+        <v>21500</v>
+      </c>
+      <c r="V76" s="21" t="n">
+        <f aca="false">V74-V75</f>
+        <v>5000</v>
+      </c>
+      <c r="W76" s="21" t="n">
+        <f aca="false">W74-W75</f>
+        <v>26500</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B77" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C77" s="21" t="n">
+        <f aca="false">C76</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="21" t="n">
+        <f aca="false">C77+D76</f>
+        <v>0</v>
+      </c>
+      <c r="E77" s="21" t="n">
+        <f aca="false">D77+E76</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="21" t="n">
+        <f aca="false">E77+F76</f>
+        <v>5000</v>
+      </c>
+      <c r="G77" s="21" t="n">
+        <f aca="false">F77+G76</f>
+        <v>5000</v>
+      </c>
+      <c r="H77" s="21" t="n">
+        <f aca="false">G77+H76</f>
+        <v>21500</v>
+      </c>
+      <c r="I77" s="21" t="n">
+        <f aca="false">H77+I76</f>
+        <v>26500</v>
+      </c>
+      <c r="J77" s="21" t="n">
+        <f aca="false">I77+J76</f>
+        <v>26500</v>
+      </c>
+      <c r="K77" s="21" t="n">
+        <f aca="false">J77+K76</f>
+        <v>26500</v>
+      </c>
+      <c r="L77" s="21" t="n">
+        <f aca="false">K77+L76</f>
+        <v>26500</v>
+      </c>
+      <c r="M77" s="21" t="n">
+        <f aca="false">L77+M76</f>
+        <v>26500</v>
+      </c>
+      <c r="N77" s="21" t="n">
+        <f aca="false">M77+N76</f>
+        <v>26500</v>
+      </c>
+      <c r="O77" s="21" t="n">
+        <f aca="false">N77+O76</f>
+        <v>26500</v>
+      </c>
+      <c r="P77" s="21" t="n">
+        <f aca="false">O77+P76</f>
+        <v>26500</v>
+      </c>
+      <c r="Q77" s="21" t="n">
+        <f aca="false">P77+Q76</f>
+        <v>26500</v>
+      </c>
+      <c r="R77" s="21" t="n">
+        <f aca="false">Q77+R76</f>
+        <v>26500</v>
+      </c>
+      <c r="S77" s="21" t="n">
+        <f aca="false">R77+S76</f>
+        <v>26500</v>
+      </c>
+      <c r="T77" s="21" t="n">
+        <f aca="false">S77+T76</f>
+        <v>26500</v>
+      </c>
+      <c r="U77" s="21" t="n">
+        <f aca="false">H77</f>
+        <v>21500</v>
+      </c>
+      <c r="V77" s="21" t="n">
+        <f aca="false">T77</f>
+        <v>26500</v>
+      </c>
+      <c r="W77" s="21" t="n">
+        <f aca="false">T77</f>
+        <v>26500</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="23"/>
+      <c r="B81" s="24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="25"/>
+      <c r="B82" s="24" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="26"/>
+      <c r="B83" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="27" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C9:W45">
+  <conditionalFormatting sqref="C8:W77">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C44:W45">
+  <conditionalFormatting sqref="C76:W77">
     <cfRule type="cellIs" priority="3" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -3954,124 +5104,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">Cashflow!U42</f>
-        <v>0</v>
+        <f aca="false">Cashflow!U74</f>
+        <v>36500</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B8" s="11" t="n">
-        <f aca="false">Cashflow!U43</f>
-        <v>0</v>
+        <f aca="false">Cashflow!U75</f>
+        <v>15000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B9" s="21" t="n">
-        <f aca="false">Cashflow!U44</f>
-        <v>0</v>
+        <f aca="false">Cashflow!U76</f>
+        <v>21500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B11" s="11" t="n">
-        <f aca="false">Cashflow!V42</f>
-        <v>0</v>
+        <f aca="false">Cashflow!V74</f>
+        <v>20000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B12" s="11" t="n">
-        <f aca="false">Cashflow!V43</f>
-        <v>0</v>
+        <f aca="false">Cashflow!V75</f>
+        <v>15000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B13" s="21" t="n">
-        <f aca="false">Cashflow!V44</f>
-        <v>0</v>
+        <f aca="false">Cashflow!V76</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="B14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">Cashflow!W42</f>
-        <v>0</v>
+        <f aca="false">Cashflow!W74</f>
+        <v>56500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B16" s="11" t="n">
-        <f aca="false">Cashflow!W43</f>
-        <v>0</v>
+        <f aca="false">Cashflow!W75</f>
+        <v>30000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B17" s="21" t="n">
-        <f aca="false">Cashflow!W44</f>
-        <v>0</v>
+        <f aca="false">Cashflow!W76</f>
+        <v>26500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Put the order number first on the order sheet
Reorders the Aufträge columns to Auftrag, Themenfeld, Kategorie,
Kostenstelle, dates, amounts, probability, so the key of each row reads
first — matching how the Cashflow sheet leads with its position column.

- Auftrag column widened and styled like the Cashflow position column
- Freeze pane and print titles now keep the Auftrag column in view
- Dropdowns follow their columns to B and C

Cashflow formulas address the table by column name, so the aggregation is
unaffected; verified end to end after the change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USZ2QFd3neqnzoYuSHpCqM
</commit_message>
<xml_diff>
--- a/deliverables/cashflow/Cashflow_SmartInfra_IoT_DusL_Plus_Autostrom_2026_2027.xlsx
+++ b/deliverables/cashflow/Cashflow_SmartInfra_IoT_DusL_Plus_Autostrom_2026_2027.xlsx
@@ -14,10 +14,11 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Aufträge!$A$1:$I$156</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Aufträge!$6:$6</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Aufträge!$A:$A,Aufträge!$6:$6</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Cashflow!$A$1:$Y$184</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$A:$D,Cashflow!$6:$6</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Cashflow!$6:$6,Cashflow!$A:$D</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Aufträge!$6:$6,Aufträge!$A:$A</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -612,7 +613,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -731,6 +732,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1318,11 +1323,11 @@
         </c:ser>
         <c:gapWidth val="40"/>
         <c:overlap val="0"/>
-        <c:axId val="26784114"/>
-        <c:axId val="86750637"/>
+        <c:axId val="94335716"/>
+        <c:axId val="88127246"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="26784114"/>
+        <c:axId val="94335716"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1354,7 +1359,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86750637"/>
+        <c:crossAx val="88127246"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1362,7 +1367,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86750637"/>
+        <c:axId val="88127246"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1438,7 +1443,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26784114"/>
+        <c:crossAx val="94335716"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1903,11 +1908,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="52973330"/>
-        <c:axId val="78151108"/>
+        <c:axId val="72081736"/>
+        <c:axId val="71250494"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52973330"/>
+        <c:axId val="72081736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1939,7 +1944,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78151108"/>
+        <c:crossAx val="71250494"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1947,7 +1952,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78151108"/>
+        <c:axId val="71250494"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2023,7 +2028,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52973330"/>
+        <c:crossAx val="72081736"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2144,9 +2149,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblAuftraege" displayName="tblAuftraege" ref="A6:I156" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A6:I156"/>
   <tableColumns count="9">
-    <tableColumn id="1" name="Themenfeld"/>
-    <tableColumn id="2" name="Kategorie"/>
-    <tableColumn id="3" name="Auftrag"/>
+    <tableColumn id="1" name="Auftrag"/>
+    <tableColumn id="2" name="Themenfeld"/>
+    <tableColumn id="3" name="Kategorie"/>
     <tableColumn id="4" name="Kostenstelle"/>
     <tableColumn id="5" name="Datum Einnahmen"/>
     <tableColumn id="6" name="Datum Ausgaben"/>
@@ -17660,10 +17665,10 @@
   <dimension ref="A1:I156"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
@@ -17690,16 +17695,16 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E6" s="6" t="s">
@@ -17720,1661 +17725,1661 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="33"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="34"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="30"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="33"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="33"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="34"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="30"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="33"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="34"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="33"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="33"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="34"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="33"/>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="34"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="33"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="33"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="34"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="33"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="33"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="34"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="33"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="33"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="33"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="30"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="33"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="33"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="30"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="33"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="34"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="30"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="33"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="30"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="34"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="30"/>
-      <c r="B27" s="30"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="33"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="34"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30"/>
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="32"/>
-      <c r="I29" s="33"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="34"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="30"/>
-      <c r="B31" s="30"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="33"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="30"/>
-      <c r="B32" s="30"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
-      <c r="I32" s="33"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="34"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="33"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="32"/>
-      <c r="I34" s="33"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="34"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="33"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="30"/>
-      <c r="B36" s="30"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="33"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="34"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="30"/>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="33"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="34"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="30"/>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="33"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="33"/>
+      <c r="I38" s="34"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="30"/>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="31"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="33"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="34"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="33"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="33"/>
+      <c r="I40" s="34"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="32"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="33"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="34"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="30"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="33"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="34"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="30"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="33"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="34"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="30"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="31"/>
-      <c r="F44" s="31"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="33"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="33"/>
+      <c r="I44" s="34"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="30"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="33"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="34"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="30"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="31"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="32"/>
-      <c r="H46" s="32"/>
-      <c r="I46" s="33"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="33"/>
+      <c r="H46" s="33"/>
+      <c r="I46" s="34"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="30"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="31"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="33"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="34"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="30"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="31"/>
-      <c r="F48" s="31"/>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="33"/>
+      <c r="B48" s="31"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="34"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="30"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="31"/>
-      <c r="F49" s="31"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="33"/>
+      <c r="B49" s="31"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="33"/>
+      <c r="I49" s="34"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="30"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="31"/>
-      <c r="F50" s="31"/>
-      <c r="G50" s="32"/>
-      <c r="H50" s="32"/>
-      <c r="I50" s="33"/>
+      <c r="B50" s="31"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="31"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="33"/>
+      <c r="I50" s="34"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="30"/>
-      <c r="B51" s="30"/>
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
-      <c r="E51" s="31"/>
-      <c r="F51" s="31"/>
-      <c r="G51" s="32"/>
-      <c r="H51" s="32"/>
-      <c r="I51" s="33"/>
+      <c r="B51" s="31"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="33"/>
+      <c r="I51" s="34"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="30"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="32"/>
-      <c r="I52" s="33"/>
+      <c r="B52" s="31"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="31"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="33"/>
+      <c r="H52" s="33"/>
+      <c r="I52" s="34"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="30"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="31"/>
-      <c r="F53" s="31"/>
-      <c r="G53" s="32"/>
-      <c r="H53" s="32"/>
-      <c r="I53" s="33"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="33"/>
+      <c r="H53" s="33"/>
+      <c r="I53" s="34"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="30"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="31"/>
-      <c r="F54" s="31"/>
-      <c r="G54" s="32"/>
-      <c r="H54" s="32"/>
-      <c r="I54" s="33"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="31"/>
+      <c r="E54" s="32"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="33"/>
+      <c r="H54" s="33"/>
+      <c r="I54" s="34"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="30"/>
-      <c r="B55" s="30"/>
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
-      <c r="E55" s="31"/>
-      <c r="F55" s="31"/>
-      <c r="G55" s="32"/>
-      <c r="H55" s="32"/>
-      <c r="I55" s="33"/>
+      <c r="B55" s="31"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="31"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="33"/>
+      <c r="H55" s="33"/>
+      <c r="I55" s="34"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="30"/>
-      <c r="B56" s="30"/>
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="31"/>
-      <c r="F56" s="31"/>
-      <c r="G56" s="32"/>
-      <c r="H56" s="32"/>
-      <c r="I56" s="33"/>
+      <c r="B56" s="31"/>
+      <c r="C56" s="31"/>
+      <c r="D56" s="31"/>
+      <c r="E56" s="32"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="33"/>
+      <c r="H56" s="33"/>
+      <c r="I56" s="34"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="30"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="30"/>
-      <c r="D57" s="30"/>
-      <c r="E57" s="31"/>
-      <c r="F57" s="31"/>
-      <c r="G57" s="32"/>
-      <c r="H57" s="32"/>
-      <c r="I57" s="33"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="32"/>
+      <c r="F57" s="32"/>
+      <c r="G57" s="33"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="34"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="30"/>
-      <c r="B58" s="30"/>
-      <c r="C58" s="30"/>
-      <c r="D58" s="30"/>
-      <c r="E58" s="31"/>
-      <c r="F58" s="31"/>
-      <c r="G58" s="32"/>
-      <c r="H58" s="32"/>
-      <c r="I58" s="33"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="31"/>
+      <c r="E58" s="32"/>
+      <c r="F58" s="32"/>
+      <c r="G58" s="33"/>
+      <c r="H58" s="33"/>
+      <c r="I58" s="34"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="30"/>
-      <c r="B59" s="30"/>
-      <c r="C59" s="30"/>
-      <c r="D59" s="30"/>
-      <c r="E59" s="31"/>
-      <c r="F59" s="31"/>
-      <c r="G59" s="32"/>
-      <c r="H59" s="32"/>
-      <c r="I59" s="33"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="31"/>
+      <c r="E59" s="32"/>
+      <c r="F59" s="32"/>
+      <c r="G59" s="33"/>
+      <c r="H59" s="33"/>
+      <c r="I59" s="34"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="30"/>
-      <c r="B60" s="30"/>
-      <c r="C60" s="30"/>
-      <c r="D60" s="30"/>
-      <c r="E60" s="31"/>
-      <c r="F60" s="31"/>
-      <c r="G60" s="32"/>
-      <c r="H60" s="32"/>
-      <c r="I60" s="33"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="31"/>
+      <c r="E60" s="32"/>
+      <c r="F60" s="32"/>
+      <c r="G60" s="33"/>
+      <c r="H60" s="33"/>
+      <c r="I60" s="34"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="30"/>
-      <c r="B61" s="30"/>
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
-      <c r="E61" s="31"/>
-      <c r="F61" s="31"/>
-      <c r="G61" s="32"/>
-      <c r="H61" s="32"/>
-      <c r="I61" s="33"/>
+      <c r="B61" s="31"/>
+      <c r="C61" s="31"/>
+      <c r="D61" s="31"/>
+      <c r="E61" s="32"/>
+      <c r="F61" s="32"/>
+      <c r="G61" s="33"/>
+      <c r="H61" s="33"/>
+      <c r="I61" s="34"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="30"/>
-      <c r="B62" s="30"/>
-      <c r="C62" s="30"/>
-      <c r="D62" s="30"/>
-      <c r="E62" s="31"/>
-      <c r="F62" s="31"/>
-      <c r="G62" s="32"/>
-      <c r="H62" s="32"/>
-      <c r="I62" s="33"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="31"/>
+      <c r="E62" s="32"/>
+      <c r="F62" s="32"/>
+      <c r="G62" s="33"/>
+      <c r="H62" s="33"/>
+      <c r="I62" s="34"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="30"/>
-      <c r="B63" s="30"/>
-      <c r="C63" s="30"/>
-      <c r="D63" s="30"/>
-      <c r="E63" s="31"/>
-      <c r="F63" s="31"/>
-      <c r="G63" s="32"/>
-      <c r="H63" s="32"/>
-      <c r="I63" s="33"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="32"/>
+      <c r="F63" s="32"/>
+      <c r="G63" s="33"/>
+      <c r="H63" s="33"/>
+      <c r="I63" s="34"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="30"/>
-      <c r="B64" s="30"/>
-      <c r="C64" s="30"/>
-      <c r="D64" s="30"/>
-      <c r="E64" s="31"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="32"/>
-      <c r="H64" s="32"/>
-      <c r="I64" s="33"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="31"/>
+      <c r="E64" s="32"/>
+      <c r="F64" s="32"/>
+      <c r="G64" s="33"/>
+      <c r="H64" s="33"/>
+      <c r="I64" s="34"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="30"/>
-      <c r="B65" s="30"/>
-      <c r="C65" s="30"/>
-      <c r="D65" s="30"/>
-      <c r="E65" s="31"/>
-      <c r="F65" s="31"/>
-      <c r="G65" s="32"/>
-      <c r="H65" s="32"/>
-      <c r="I65" s="33"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="E65" s="32"/>
+      <c r="F65" s="32"/>
+      <c r="G65" s="33"/>
+      <c r="H65" s="33"/>
+      <c r="I65" s="34"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="30"/>
-      <c r="B66" s="30"/>
-      <c r="C66" s="30"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="31"/>
-      <c r="F66" s="31"/>
-      <c r="G66" s="32"/>
-      <c r="H66" s="32"/>
-      <c r="I66" s="33"/>
+      <c r="B66" s="31"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="E66" s="32"/>
+      <c r="F66" s="32"/>
+      <c r="G66" s="33"/>
+      <c r="H66" s="33"/>
+      <c r="I66" s="34"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="30"/>
-      <c r="B67" s="30"/>
-      <c r="C67" s="30"/>
-      <c r="D67" s="30"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="32"/>
-      <c r="H67" s="32"/>
-      <c r="I67" s="33"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="32"/>
+      <c r="F67" s="32"/>
+      <c r="G67" s="33"/>
+      <c r="H67" s="33"/>
+      <c r="I67" s="34"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="30"/>
-      <c r="B68" s="30"/>
-      <c r="C68" s="30"/>
-      <c r="D68" s="30"/>
-      <c r="E68" s="31"/>
-      <c r="F68" s="31"/>
-      <c r="G68" s="32"/>
-      <c r="H68" s="32"/>
-      <c r="I68" s="33"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="31"/>
+      <c r="D68" s="31"/>
+      <c r="E68" s="32"/>
+      <c r="F68" s="32"/>
+      <c r="G68" s="33"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="34"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="30"/>
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="30"/>
-      <c r="E69" s="31"/>
-      <c r="F69" s="31"/>
-      <c r="G69" s="32"/>
-      <c r="H69" s="32"/>
-      <c r="I69" s="33"/>
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="32"/>
+      <c r="F69" s="32"/>
+      <c r="G69" s="33"/>
+      <c r="H69" s="33"/>
+      <c r="I69" s="34"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="30"/>
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
-      <c r="D70" s="30"/>
-      <c r="E70" s="31"/>
-      <c r="F70" s="31"/>
-      <c r="G70" s="32"/>
-      <c r="H70" s="32"/>
-      <c r="I70" s="33"/>
+      <c r="B70" s="31"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="32"/>
+      <c r="F70" s="32"/>
+      <c r="G70" s="33"/>
+      <c r="H70" s="33"/>
+      <c r="I70" s="34"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="30"/>
-      <c r="B71" s="30"/>
-      <c r="C71" s="30"/>
-      <c r="D71" s="30"/>
-      <c r="E71" s="31"/>
-      <c r="F71" s="31"/>
-      <c r="G71" s="32"/>
-      <c r="H71" s="32"/>
-      <c r="I71" s="33"/>
+      <c r="B71" s="31"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="31"/>
+      <c r="E71" s="32"/>
+      <c r="F71" s="32"/>
+      <c r="G71" s="33"/>
+      <c r="H71" s="33"/>
+      <c r="I71" s="34"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="30"/>
-      <c r="B72" s="30"/>
-      <c r="C72" s="30"/>
-      <c r="D72" s="30"/>
-      <c r="E72" s="31"/>
-      <c r="F72" s="31"/>
-      <c r="G72" s="32"/>
-      <c r="H72" s="32"/>
-      <c r="I72" s="33"/>
+      <c r="B72" s="31"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="32"/>
+      <c r="F72" s="32"/>
+      <c r="G72" s="33"/>
+      <c r="H72" s="33"/>
+      <c r="I72" s="34"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="30"/>
-      <c r="B73" s="30"/>
-      <c r="C73" s="30"/>
-      <c r="D73" s="30"/>
-      <c r="E73" s="31"/>
-      <c r="F73" s="31"/>
-      <c r="G73" s="32"/>
-      <c r="H73" s="32"/>
-      <c r="I73" s="33"/>
+      <c r="B73" s="31"/>
+      <c r="C73" s="31"/>
+      <c r="D73" s="31"/>
+      <c r="E73" s="32"/>
+      <c r="F73" s="32"/>
+      <c r="G73" s="33"/>
+      <c r="H73" s="33"/>
+      <c r="I73" s="34"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="30"/>
-      <c r="B74" s="30"/>
-      <c r="C74" s="30"/>
-      <c r="D74" s="30"/>
-      <c r="E74" s="31"/>
-      <c r="F74" s="31"/>
-      <c r="G74" s="32"/>
-      <c r="H74" s="32"/>
-      <c r="I74" s="33"/>
+      <c r="B74" s="31"/>
+      <c r="C74" s="31"/>
+      <c r="D74" s="31"/>
+      <c r="E74" s="32"/>
+      <c r="F74" s="32"/>
+      <c r="G74" s="33"/>
+      <c r="H74" s="33"/>
+      <c r="I74" s="34"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="30"/>
-      <c r="B75" s="30"/>
-      <c r="C75" s="30"/>
-      <c r="D75" s="30"/>
-      <c r="E75" s="31"/>
-      <c r="F75" s="31"/>
-      <c r="G75" s="32"/>
-      <c r="H75" s="32"/>
-      <c r="I75" s="33"/>
+      <c r="B75" s="31"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="31"/>
+      <c r="E75" s="32"/>
+      <c r="F75" s="32"/>
+      <c r="G75" s="33"/>
+      <c r="H75" s="33"/>
+      <c r="I75" s="34"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="30"/>
-      <c r="B76" s="30"/>
-      <c r="C76" s="30"/>
-      <c r="D76" s="30"/>
-      <c r="E76" s="31"/>
-      <c r="F76" s="31"/>
-      <c r="G76" s="32"/>
-      <c r="H76" s="32"/>
-      <c r="I76" s="33"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="32"/>
+      <c r="F76" s="32"/>
+      <c r="G76" s="33"/>
+      <c r="H76" s="33"/>
+      <c r="I76" s="34"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="30"/>
-      <c r="B77" s="30"/>
-      <c r="C77" s="30"/>
-      <c r="D77" s="30"/>
-      <c r="E77" s="31"/>
-      <c r="F77" s="31"/>
-      <c r="G77" s="32"/>
-      <c r="H77" s="32"/>
-      <c r="I77" s="33"/>
+      <c r="B77" s="31"/>
+      <c r="C77" s="31"/>
+      <c r="D77" s="31"/>
+      <c r="E77" s="32"/>
+      <c r="F77" s="32"/>
+      <c r="G77" s="33"/>
+      <c r="H77" s="33"/>
+      <c r="I77" s="34"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="30"/>
-      <c r="B78" s="30"/>
-      <c r="C78" s="30"/>
-      <c r="D78" s="30"/>
-      <c r="E78" s="31"/>
-      <c r="F78" s="31"/>
-      <c r="G78" s="32"/>
-      <c r="H78" s="32"/>
-      <c r="I78" s="33"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="32"/>
+      <c r="F78" s="32"/>
+      <c r="G78" s="33"/>
+      <c r="H78" s="33"/>
+      <c r="I78" s="34"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="30"/>
-      <c r="B79" s="30"/>
-      <c r="C79" s="30"/>
-      <c r="D79" s="30"/>
-      <c r="E79" s="31"/>
-      <c r="F79" s="31"/>
-      <c r="G79" s="32"/>
-      <c r="H79" s="32"/>
-      <c r="I79" s="33"/>
+      <c r="B79" s="31"/>
+      <c r="C79" s="31"/>
+      <c r="D79" s="31"/>
+      <c r="E79" s="32"/>
+      <c r="F79" s="32"/>
+      <c r="G79" s="33"/>
+      <c r="H79" s="33"/>
+      <c r="I79" s="34"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="30"/>
-      <c r="B80" s="30"/>
-      <c r="C80" s="30"/>
-      <c r="D80" s="30"/>
-      <c r="E80" s="31"/>
-      <c r="F80" s="31"/>
-      <c r="G80" s="32"/>
-      <c r="H80" s="32"/>
-      <c r="I80" s="33"/>
+      <c r="B80" s="31"/>
+      <c r="C80" s="31"/>
+      <c r="D80" s="31"/>
+      <c r="E80" s="32"/>
+      <c r="F80" s="32"/>
+      <c r="G80" s="33"/>
+      <c r="H80" s="33"/>
+      <c r="I80" s="34"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="30"/>
-      <c r="B81" s="30"/>
-      <c r="C81" s="30"/>
-      <c r="D81" s="30"/>
-      <c r="E81" s="31"/>
-      <c r="F81" s="31"/>
-      <c r="G81" s="32"/>
-      <c r="H81" s="32"/>
-      <c r="I81" s="33"/>
+      <c r="B81" s="31"/>
+      <c r="C81" s="31"/>
+      <c r="D81" s="31"/>
+      <c r="E81" s="32"/>
+      <c r="F81" s="32"/>
+      <c r="G81" s="33"/>
+      <c r="H81" s="33"/>
+      <c r="I81" s="34"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="30"/>
-      <c r="B82" s="30"/>
-      <c r="C82" s="30"/>
-      <c r="D82" s="30"/>
-      <c r="E82" s="31"/>
-      <c r="F82" s="31"/>
-      <c r="G82" s="32"/>
-      <c r="H82" s="32"/>
-      <c r="I82" s="33"/>
+      <c r="B82" s="31"/>
+      <c r="C82" s="31"/>
+      <c r="D82" s="31"/>
+      <c r="E82" s="32"/>
+      <c r="F82" s="32"/>
+      <c r="G82" s="33"/>
+      <c r="H82" s="33"/>
+      <c r="I82" s="34"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="30"/>
-      <c r="B83" s="30"/>
-      <c r="C83" s="30"/>
-      <c r="D83" s="30"/>
-      <c r="E83" s="31"/>
-      <c r="F83" s="31"/>
-      <c r="G83" s="32"/>
-      <c r="H83" s="32"/>
-      <c r="I83" s="33"/>
+      <c r="B83" s="31"/>
+      <c r="C83" s="31"/>
+      <c r="D83" s="31"/>
+      <c r="E83" s="32"/>
+      <c r="F83" s="32"/>
+      <c r="G83" s="33"/>
+      <c r="H83" s="33"/>
+      <c r="I83" s="34"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="30"/>
-      <c r="B84" s="30"/>
-      <c r="C84" s="30"/>
-      <c r="D84" s="30"/>
-      <c r="E84" s="31"/>
-      <c r="F84" s="31"/>
-      <c r="G84" s="32"/>
-      <c r="H84" s="32"/>
-      <c r="I84" s="33"/>
+      <c r="B84" s="31"/>
+      <c r="C84" s="31"/>
+      <c r="D84" s="31"/>
+      <c r="E84" s="32"/>
+      <c r="F84" s="32"/>
+      <c r="G84" s="33"/>
+      <c r="H84" s="33"/>
+      <c r="I84" s="34"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="30"/>
-      <c r="B85" s="30"/>
-      <c r="C85" s="30"/>
-      <c r="D85" s="30"/>
-      <c r="E85" s="31"/>
-      <c r="F85" s="31"/>
-      <c r="G85" s="32"/>
-      <c r="H85" s="32"/>
-      <c r="I85" s="33"/>
+      <c r="B85" s="31"/>
+      <c r="C85" s="31"/>
+      <c r="D85" s="31"/>
+      <c r="E85" s="32"/>
+      <c r="F85" s="32"/>
+      <c r="G85" s="33"/>
+      <c r="H85" s="33"/>
+      <c r="I85" s="34"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="30"/>
-      <c r="B86" s="30"/>
-      <c r="C86" s="30"/>
-      <c r="D86" s="30"/>
-      <c r="E86" s="31"/>
-      <c r="F86" s="31"/>
-      <c r="G86" s="32"/>
-      <c r="H86" s="32"/>
-      <c r="I86" s="33"/>
+      <c r="B86" s="31"/>
+      <c r="C86" s="31"/>
+      <c r="D86" s="31"/>
+      <c r="E86" s="32"/>
+      <c r="F86" s="32"/>
+      <c r="G86" s="33"/>
+      <c r="H86" s="33"/>
+      <c r="I86" s="34"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="30"/>
-      <c r="B87" s="30"/>
-      <c r="C87" s="30"/>
-      <c r="D87" s="30"/>
-      <c r="E87" s="31"/>
-      <c r="F87" s="31"/>
-      <c r="G87" s="32"/>
-      <c r="H87" s="32"/>
-      <c r="I87" s="33"/>
+      <c r="B87" s="31"/>
+      <c r="C87" s="31"/>
+      <c r="D87" s="31"/>
+      <c r="E87" s="32"/>
+      <c r="F87" s="32"/>
+      <c r="G87" s="33"/>
+      <c r="H87" s="33"/>
+      <c r="I87" s="34"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="30"/>
-      <c r="B88" s="30"/>
-      <c r="C88" s="30"/>
-      <c r="D88" s="30"/>
-      <c r="E88" s="31"/>
-      <c r="F88" s="31"/>
-      <c r="G88" s="32"/>
-      <c r="H88" s="32"/>
-      <c r="I88" s="33"/>
+      <c r="B88" s="31"/>
+      <c r="C88" s="31"/>
+      <c r="D88" s="31"/>
+      <c r="E88" s="32"/>
+      <c r="F88" s="32"/>
+      <c r="G88" s="33"/>
+      <c r="H88" s="33"/>
+      <c r="I88" s="34"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="30"/>
-      <c r="B89" s="30"/>
-      <c r="C89" s="30"/>
-      <c r="D89" s="30"/>
-      <c r="E89" s="31"/>
-      <c r="F89" s="31"/>
-      <c r="G89" s="32"/>
-      <c r="H89" s="32"/>
-      <c r="I89" s="33"/>
+      <c r="B89" s="31"/>
+      <c r="C89" s="31"/>
+      <c r="D89" s="31"/>
+      <c r="E89" s="32"/>
+      <c r="F89" s="32"/>
+      <c r="G89" s="33"/>
+      <c r="H89" s="33"/>
+      <c r="I89" s="34"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="30"/>
-      <c r="B90" s="30"/>
-      <c r="C90" s="30"/>
-      <c r="D90" s="30"/>
-      <c r="E90" s="31"/>
-      <c r="F90" s="31"/>
-      <c r="G90" s="32"/>
-      <c r="H90" s="32"/>
-      <c r="I90" s="33"/>
+      <c r="B90" s="31"/>
+      <c r="C90" s="31"/>
+      <c r="D90" s="31"/>
+      <c r="E90" s="32"/>
+      <c r="F90" s="32"/>
+      <c r="G90" s="33"/>
+      <c r="H90" s="33"/>
+      <c r="I90" s="34"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="30"/>
-      <c r="B91" s="30"/>
-      <c r="C91" s="30"/>
-      <c r="D91" s="30"/>
-      <c r="E91" s="31"/>
-      <c r="F91" s="31"/>
-      <c r="G91" s="32"/>
-      <c r="H91" s="32"/>
-      <c r="I91" s="33"/>
+      <c r="B91" s="31"/>
+      <c r="C91" s="31"/>
+      <c r="D91" s="31"/>
+      <c r="E91" s="32"/>
+      <c r="F91" s="32"/>
+      <c r="G91" s="33"/>
+      <c r="H91" s="33"/>
+      <c r="I91" s="34"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="30"/>
-      <c r="B92" s="30"/>
-      <c r="C92" s="30"/>
-      <c r="D92" s="30"/>
-      <c r="E92" s="31"/>
-      <c r="F92" s="31"/>
-      <c r="G92" s="32"/>
-      <c r="H92" s="32"/>
-      <c r="I92" s="33"/>
+      <c r="B92" s="31"/>
+      <c r="C92" s="31"/>
+      <c r="D92" s="31"/>
+      <c r="E92" s="32"/>
+      <c r="F92" s="32"/>
+      <c r="G92" s="33"/>
+      <c r="H92" s="33"/>
+      <c r="I92" s="34"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="30"/>
-      <c r="B93" s="30"/>
-      <c r="C93" s="30"/>
-      <c r="D93" s="30"/>
-      <c r="E93" s="31"/>
-      <c r="F93" s="31"/>
-      <c r="G93" s="32"/>
-      <c r="H93" s="32"/>
-      <c r="I93" s="33"/>
+      <c r="B93" s="31"/>
+      <c r="C93" s="31"/>
+      <c r="D93" s="31"/>
+      <c r="E93" s="32"/>
+      <c r="F93" s="32"/>
+      <c r="G93" s="33"/>
+      <c r="H93" s="33"/>
+      <c r="I93" s="34"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="30"/>
-      <c r="B94" s="30"/>
-      <c r="C94" s="30"/>
-      <c r="D94" s="30"/>
-      <c r="E94" s="31"/>
-      <c r="F94" s="31"/>
-      <c r="G94" s="32"/>
-      <c r="H94" s="32"/>
-      <c r="I94" s="33"/>
+      <c r="B94" s="31"/>
+      <c r="C94" s="31"/>
+      <c r="D94" s="31"/>
+      <c r="E94" s="32"/>
+      <c r="F94" s="32"/>
+      <c r="G94" s="33"/>
+      <c r="H94" s="33"/>
+      <c r="I94" s="34"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="30"/>
-      <c r="B95" s="30"/>
-      <c r="C95" s="30"/>
-      <c r="D95" s="30"/>
-      <c r="E95" s="31"/>
-      <c r="F95" s="31"/>
-      <c r="G95" s="32"/>
-      <c r="H95" s="32"/>
-      <c r="I95" s="33"/>
+      <c r="B95" s="31"/>
+      <c r="C95" s="31"/>
+      <c r="D95" s="31"/>
+      <c r="E95" s="32"/>
+      <c r="F95" s="32"/>
+      <c r="G95" s="33"/>
+      <c r="H95" s="33"/>
+      <c r="I95" s="34"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="30"/>
-      <c r="B96" s="30"/>
-      <c r="C96" s="30"/>
-      <c r="D96" s="30"/>
-      <c r="E96" s="31"/>
-      <c r="F96" s="31"/>
-      <c r="G96" s="32"/>
-      <c r="H96" s="32"/>
-      <c r="I96" s="33"/>
+      <c r="B96" s="31"/>
+      <c r="C96" s="31"/>
+      <c r="D96" s="31"/>
+      <c r="E96" s="32"/>
+      <c r="F96" s="32"/>
+      <c r="G96" s="33"/>
+      <c r="H96" s="33"/>
+      <c r="I96" s="34"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="30"/>
-      <c r="B97" s="30"/>
-      <c r="C97" s="30"/>
-      <c r="D97" s="30"/>
-      <c r="E97" s="31"/>
-      <c r="F97" s="31"/>
-      <c r="G97" s="32"/>
-      <c r="H97" s="32"/>
-      <c r="I97" s="33"/>
+      <c r="B97" s="31"/>
+      <c r="C97" s="31"/>
+      <c r="D97" s="31"/>
+      <c r="E97" s="32"/>
+      <c r="F97" s="32"/>
+      <c r="G97" s="33"/>
+      <c r="H97" s="33"/>
+      <c r="I97" s="34"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="30"/>
-      <c r="B98" s="30"/>
-      <c r="C98" s="30"/>
-      <c r="D98" s="30"/>
-      <c r="E98" s="31"/>
-      <c r="F98" s="31"/>
-      <c r="G98" s="32"/>
-      <c r="H98" s="32"/>
-      <c r="I98" s="33"/>
+      <c r="B98" s="31"/>
+      <c r="C98" s="31"/>
+      <c r="D98" s="31"/>
+      <c r="E98" s="32"/>
+      <c r="F98" s="32"/>
+      <c r="G98" s="33"/>
+      <c r="H98" s="33"/>
+      <c r="I98" s="34"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="30"/>
-      <c r="B99" s="30"/>
-      <c r="C99" s="30"/>
-      <c r="D99" s="30"/>
-      <c r="E99" s="31"/>
-      <c r="F99" s="31"/>
-      <c r="G99" s="32"/>
-      <c r="H99" s="32"/>
-      <c r="I99" s="33"/>
+      <c r="B99" s="31"/>
+      <c r="C99" s="31"/>
+      <c r="D99" s="31"/>
+      <c r="E99" s="32"/>
+      <c r="F99" s="32"/>
+      <c r="G99" s="33"/>
+      <c r="H99" s="33"/>
+      <c r="I99" s="34"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="30"/>
-      <c r="B100" s="30"/>
-      <c r="C100" s="30"/>
-      <c r="D100" s="30"/>
-      <c r="E100" s="31"/>
-      <c r="F100" s="31"/>
-      <c r="G100" s="32"/>
-      <c r="H100" s="32"/>
-      <c r="I100" s="33"/>
+      <c r="B100" s="31"/>
+      <c r="C100" s="31"/>
+      <c r="D100" s="31"/>
+      <c r="E100" s="32"/>
+      <c r="F100" s="32"/>
+      <c r="G100" s="33"/>
+      <c r="H100" s="33"/>
+      <c r="I100" s="34"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="30"/>
-      <c r="B101" s="30"/>
-      <c r="C101" s="30"/>
-      <c r="D101" s="30"/>
-      <c r="E101" s="31"/>
-      <c r="F101" s="31"/>
-      <c r="G101" s="32"/>
-      <c r="H101" s="32"/>
-      <c r="I101" s="33"/>
+      <c r="B101" s="31"/>
+      <c r="C101" s="31"/>
+      <c r="D101" s="31"/>
+      <c r="E101" s="32"/>
+      <c r="F101" s="32"/>
+      <c r="G101" s="33"/>
+      <c r="H101" s="33"/>
+      <c r="I101" s="34"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="30"/>
-      <c r="B102" s="30"/>
-      <c r="C102" s="30"/>
-      <c r="D102" s="30"/>
-      <c r="E102" s="31"/>
-      <c r="F102" s="31"/>
-      <c r="G102" s="32"/>
-      <c r="H102" s="32"/>
-      <c r="I102" s="33"/>
+      <c r="B102" s="31"/>
+      <c r="C102" s="31"/>
+      <c r="D102" s="31"/>
+      <c r="E102" s="32"/>
+      <c r="F102" s="32"/>
+      <c r="G102" s="33"/>
+      <c r="H102" s="33"/>
+      <c r="I102" s="34"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="30"/>
-      <c r="B103" s="30"/>
-      <c r="C103" s="30"/>
-      <c r="D103" s="30"/>
-      <c r="E103" s="31"/>
-      <c r="F103" s="31"/>
-      <c r="G103" s="32"/>
-      <c r="H103" s="32"/>
-      <c r="I103" s="33"/>
+      <c r="B103" s="31"/>
+      <c r="C103" s="31"/>
+      <c r="D103" s="31"/>
+      <c r="E103" s="32"/>
+      <c r="F103" s="32"/>
+      <c r="G103" s="33"/>
+      <c r="H103" s="33"/>
+      <c r="I103" s="34"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="30"/>
-      <c r="B104" s="30"/>
-      <c r="C104" s="30"/>
-      <c r="D104" s="30"/>
-      <c r="E104" s="31"/>
-      <c r="F104" s="31"/>
-      <c r="G104" s="32"/>
-      <c r="H104" s="32"/>
-      <c r="I104" s="33"/>
+      <c r="B104" s="31"/>
+      <c r="C104" s="31"/>
+      <c r="D104" s="31"/>
+      <c r="E104" s="32"/>
+      <c r="F104" s="32"/>
+      <c r="G104" s="33"/>
+      <c r="H104" s="33"/>
+      <c r="I104" s="34"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="30"/>
-      <c r="B105" s="30"/>
-      <c r="C105" s="30"/>
-      <c r="D105" s="30"/>
-      <c r="E105" s="31"/>
-      <c r="F105" s="31"/>
-      <c r="G105" s="32"/>
-      <c r="H105" s="32"/>
-      <c r="I105" s="33"/>
+      <c r="B105" s="31"/>
+      <c r="C105" s="31"/>
+      <c r="D105" s="31"/>
+      <c r="E105" s="32"/>
+      <c r="F105" s="32"/>
+      <c r="G105" s="33"/>
+      <c r="H105" s="33"/>
+      <c r="I105" s="34"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="30"/>
-      <c r="B106" s="30"/>
-      <c r="C106" s="30"/>
-      <c r="D106" s="30"/>
-      <c r="E106" s="31"/>
-      <c r="F106" s="31"/>
-      <c r="G106" s="32"/>
-      <c r="H106" s="32"/>
-      <c r="I106" s="33"/>
+      <c r="B106" s="31"/>
+      <c r="C106" s="31"/>
+      <c r="D106" s="31"/>
+      <c r="E106" s="32"/>
+      <c r="F106" s="32"/>
+      <c r="G106" s="33"/>
+      <c r="H106" s="33"/>
+      <c r="I106" s="34"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="30"/>
-      <c r="B107" s="30"/>
-      <c r="C107" s="30"/>
-      <c r="D107" s="30"/>
-      <c r="E107" s="31"/>
-      <c r="F107" s="31"/>
-      <c r="G107" s="32"/>
-      <c r="H107" s="32"/>
-      <c r="I107" s="33"/>
+      <c r="B107" s="31"/>
+      <c r="C107" s="31"/>
+      <c r="D107" s="31"/>
+      <c r="E107" s="32"/>
+      <c r="F107" s="32"/>
+      <c r="G107" s="33"/>
+      <c r="H107" s="33"/>
+      <c r="I107" s="34"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="30"/>
-      <c r="B108" s="30"/>
-      <c r="C108" s="30"/>
-      <c r="D108" s="30"/>
-      <c r="E108" s="31"/>
-      <c r="F108" s="31"/>
-      <c r="G108" s="32"/>
-      <c r="H108" s="32"/>
-      <c r="I108" s="33"/>
+      <c r="B108" s="31"/>
+      <c r="C108" s="31"/>
+      <c r="D108" s="31"/>
+      <c r="E108" s="32"/>
+      <c r="F108" s="32"/>
+      <c r="G108" s="33"/>
+      <c r="H108" s="33"/>
+      <c r="I108" s="34"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="30"/>
-      <c r="B109" s="30"/>
-      <c r="C109" s="30"/>
-      <c r="D109" s="30"/>
-      <c r="E109" s="31"/>
-      <c r="F109" s="31"/>
-      <c r="G109" s="32"/>
-      <c r="H109" s="32"/>
-      <c r="I109" s="33"/>
+      <c r="B109" s="31"/>
+      <c r="C109" s="31"/>
+      <c r="D109" s="31"/>
+      <c r="E109" s="32"/>
+      <c r="F109" s="32"/>
+      <c r="G109" s="33"/>
+      <c r="H109" s="33"/>
+      <c r="I109" s="34"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="30"/>
-      <c r="B110" s="30"/>
-      <c r="C110" s="30"/>
-      <c r="D110" s="30"/>
-      <c r="E110" s="31"/>
-      <c r="F110" s="31"/>
-      <c r="G110" s="32"/>
-      <c r="H110" s="32"/>
-      <c r="I110" s="33"/>
+      <c r="B110" s="31"/>
+      <c r="C110" s="31"/>
+      <c r="D110" s="31"/>
+      <c r="E110" s="32"/>
+      <c r="F110" s="32"/>
+      <c r="G110" s="33"/>
+      <c r="H110" s="33"/>
+      <c r="I110" s="34"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="30"/>
-      <c r="B111" s="30"/>
-      <c r="C111" s="30"/>
-      <c r="D111" s="30"/>
-      <c r="E111" s="31"/>
-      <c r="F111" s="31"/>
-      <c r="G111" s="32"/>
-      <c r="H111" s="32"/>
-      <c r="I111" s="33"/>
+      <c r="B111" s="31"/>
+      <c r="C111" s="31"/>
+      <c r="D111" s="31"/>
+      <c r="E111" s="32"/>
+      <c r="F111" s="32"/>
+      <c r="G111" s="33"/>
+      <c r="H111" s="33"/>
+      <c r="I111" s="34"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="30"/>
-      <c r="B112" s="30"/>
-      <c r="C112" s="30"/>
-      <c r="D112" s="30"/>
-      <c r="E112" s="31"/>
-      <c r="F112" s="31"/>
-      <c r="G112" s="32"/>
-      <c r="H112" s="32"/>
-      <c r="I112" s="33"/>
+      <c r="B112" s="31"/>
+      <c r="C112" s="31"/>
+      <c r="D112" s="31"/>
+      <c r="E112" s="32"/>
+      <c r="F112" s="32"/>
+      <c r="G112" s="33"/>
+      <c r="H112" s="33"/>
+      <c r="I112" s="34"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="30"/>
-      <c r="B113" s="30"/>
-      <c r="C113" s="30"/>
-      <c r="D113" s="30"/>
-      <c r="E113" s="31"/>
-      <c r="F113" s="31"/>
-      <c r="G113" s="32"/>
-      <c r="H113" s="32"/>
-      <c r="I113" s="33"/>
+      <c r="B113" s="31"/>
+      <c r="C113" s="31"/>
+      <c r="D113" s="31"/>
+      <c r="E113" s="32"/>
+      <c r="F113" s="32"/>
+      <c r="G113" s="33"/>
+      <c r="H113" s="33"/>
+      <c r="I113" s="34"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="30"/>
-      <c r="B114" s="30"/>
-      <c r="C114" s="30"/>
-      <c r="D114" s="30"/>
-      <c r="E114" s="31"/>
-      <c r="F114" s="31"/>
-      <c r="G114" s="32"/>
-      <c r="H114" s="32"/>
-      <c r="I114" s="33"/>
+      <c r="B114" s="31"/>
+      <c r="C114" s="31"/>
+      <c r="D114" s="31"/>
+      <c r="E114" s="32"/>
+      <c r="F114" s="32"/>
+      <c r="G114" s="33"/>
+      <c r="H114" s="33"/>
+      <c r="I114" s="34"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="30"/>
-      <c r="B115" s="30"/>
-      <c r="C115" s="30"/>
-      <c r="D115" s="30"/>
-      <c r="E115" s="31"/>
-      <c r="F115" s="31"/>
-      <c r="G115" s="32"/>
-      <c r="H115" s="32"/>
-      <c r="I115" s="33"/>
+      <c r="B115" s="31"/>
+      <c r="C115" s="31"/>
+      <c r="D115" s="31"/>
+      <c r="E115" s="32"/>
+      <c r="F115" s="32"/>
+      <c r="G115" s="33"/>
+      <c r="H115" s="33"/>
+      <c r="I115" s="34"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="30"/>
-      <c r="B116" s="30"/>
-      <c r="C116" s="30"/>
-      <c r="D116" s="30"/>
-      <c r="E116" s="31"/>
-      <c r="F116" s="31"/>
-      <c r="G116" s="32"/>
-      <c r="H116" s="32"/>
-      <c r="I116" s="33"/>
+      <c r="B116" s="31"/>
+      <c r="C116" s="31"/>
+      <c r="D116" s="31"/>
+      <c r="E116" s="32"/>
+      <c r="F116" s="32"/>
+      <c r="G116" s="33"/>
+      <c r="H116" s="33"/>
+      <c r="I116" s="34"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="30"/>
-      <c r="B117" s="30"/>
-      <c r="C117" s="30"/>
-      <c r="D117" s="30"/>
-      <c r="E117" s="31"/>
-      <c r="F117" s="31"/>
-      <c r="G117" s="32"/>
-      <c r="H117" s="32"/>
-      <c r="I117" s="33"/>
+      <c r="B117" s="31"/>
+      <c r="C117" s="31"/>
+      <c r="D117" s="31"/>
+      <c r="E117" s="32"/>
+      <c r="F117" s="32"/>
+      <c r="G117" s="33"/>
+      <c r="H117" s="33"/>
+      <c r="I117" s="34"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="30"/>
-      <c r="B118" s="30"/>
-      <c r="C118" s="30"/>
-      <c r="D118" s="30"/>
-      <c r="E118" s="31"/>
-      <c r="F118" s="31"/>
-      <c r="G118" s="32"/>
-      <c r="H118" s="32"/>
-      <c r="I118" s="33"/>
+      <c r="B118" s="31"/>
+      <c r="C118" s="31"/>
+      <c r="D118" s="31"/>
+      <c r="E118" s="32"/>
+      <c r="F118" s="32"/>
+      <c r="G118" s="33"/>
+      <c r="H118" s="33"/>
+      <c r="I118" s="34"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="30"/>
-      <c r="B119" s="30"/>
-      <c r="C119" s="30"/>
-      <c r="D119" s="30"/>
-      <c r="E119" s="31"/>
-      <c r="F119" s="31"/>
-      <c r="G119" s="32"/>
-      <c r="H119" s="32"/>
-      <c r="I119" s="33"/>
+      <c r="B119" s="31"/>
+      <c r="C119" s="31"/>
+      <c r="D119" s="31"/>
+      <c r="E119" s="32"/>
+      <c r="F119" s="32"/>
+      <c r="G119" s="33"/>
+      <c r="H119" s="33"/>
+      <c r="I119" s="34"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="30"/>
-      <c r="B120" s="30"/>
-      <c r="C120" s="30"/>
-      <c r="D120" s="30"/>
-      <c r="E120" s="31"/>
-      <c r="F120" s="31"/>
-      <c r="G120" s="32"/>
-      <c r="H120" s="32"/>
-      <c r="I120" s="33"/>
+      <c r="B120" s="31"/>
+      <c r="C120" s="31"/>
+      <c r="D120" s="31"/>
+      <c r="E120" s="32"/>
+      <c r="F120" s="32"/>
+      <c r="G120" s="33"/>
+      <c r="H120" s="33"/>
+      <c r="I120" s="34"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="30"/>
-      <c r="B121" s="30"/>
-      <c r="C121" s="30"/>
-      <c r="D121" s="30"/>
-      <c r="E121" s="31"/>
-      <c r="F121" s="31"/>
-      <c r="G121" s="32"/>
-      <c r="H121" s="32"/>
-      <c r="I121" s="33"/>
+      <c r="B121" s="31"/>
+      <c r="C121" s="31"/>
+      <c r="D121" s="31"/>
+      <c r="E121" s="32"/>
+      <c r="F121" s="32"/>
+      <c r="G121" s="33"/>
+      <c r="H121" s="33"/>
+      <c r="I121" s="34"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="30"/>
-      <c r="B122" s="30"/>
-      <c r="C122" s="30"/>
-      <c r="D122" s="30"/>
-      <c r="E122" s="31"/>
-      <c r="F122" s="31"/>
-      <c r="G122" s="32"/>
-      <c r="H122" s="32"/>
-      <c r="I122" s="33"/>
+      <c r="B122" s="31"/>
+      <c r="C122" s="31"/>
+      <c r="D122" s="31"/>
+      <c r="E122" s="32"/>
+      <c r="F122" s="32"/>
+      <c r="G122" s="33"/>
+      <c r="H122" s="33"/>
+      <c r="I122" s="34"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="30"/>
-      <c r="B123" s="30"/>
-      <c r="C123" s="30"/>
-      <c r="D123" s="30"/>
-      <c r="E123" s="31"/>
-      <c r="F123" s="31"/>
-      <c r="G123" s="32"/>
-      <c r="H123" s="32"/>
-      <c r="I123" s="33"/>
+      <c r="B123" s="31"/>
+      <c r="C123" s="31"/>
+      <c r="D123" s="31"/>
+      <c r="E123" s="32"/>
+      <c r="F123" s="32"/>
+      <c r="G123" s="33"/>
+      <c r="H123" s="33"/>
+      <c r="I123" s="34"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="30"/>
-      <c r="B124" s="30"/>
-      <c r="C124" s="30"/>
-      <c r="D124" s="30"/>
-      <c r="E124" s="31"/>
-      <c r="F124" s="31"/>
-      <c r="G124" s="32"/>
-      <c r="H124" s="32"/>
-      <c r="I124" s="33"/>
+      <c r="B124" s="31"/>
+      <c r="C124" s="31"/>
+      <c r="D124" s="31"/>
+      <c r="E124" s="32"/>
+      <c r="F124" s="32"/>
+      <c r="G124" s="33"/>
+      <c r="H124" s="33"/>
+      <c r="I124" s="34"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="30"/>
-      <c r="B125" s="30"/>
-      <c r="C125" s="30"/>
-      <c r="D125" s="30"/>
-      <c r="E125" s="31"/>
-      <c r="F125" s="31"/>
-      <c r="G125" s="32"/>
-      <c r="H125" s="32"/>
-      <c r="I125" s="33"/>
+      <c r="B125" s="31"/>
+      <c r="C125" s="31"/>
+      <c r="D125" s="31"/>
+      <c r="E125" s="32"/>
+      <c r="F125" s="32"/>
+      <c r="G125" s="33"/>
+      <c r="H125" s="33"/>
+      <c r="I125" s="34"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="30"/>
-      <c r="B126" s="30"/>
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
-      <c r="E126" s="31"/>
-      <c r="F126" s="31"/>
-      <c r="G126" s="32"/>
-      <c r="H126" s="32"/>
-      <c r="I126" s="33"/>
+      <c r="B126" s="31"/>
+      <c r="C126" s="31"/>
+      <c r="D126" s="31"/>
+      <c r="E126" s="32"/>
+      <c r="F126" s="32"/>
+      <c r="G126" s="33"/>
+      <c r="H126" s="33"/>
+      <c r="I126" s="34"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="30"/>
-      <c r="B127" s="30"/>
-      <c r="C127" s="30"/>
-      <c r="D127" s="30"/>
-      <c r="E127" s="31"/>
-      <c r="F127" s="31"/>
-      <c r="G127" s="32"/>
-      <c r="H127" s="32"/>
-      <c r="I127" s="33"/>
+      <c r="B127" s="31"/>
+      <c r="C127" s="31"/>
+      <c r="D127" s="31"/>
+      <c r="E127" s="32"/>
+      <c r="F127" s="32"/>
+      <c r="G127" s="33"/>
+      <c r="H127" s="33"/>
+      <c r="I127" s="34"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="30"/>
-      <c r="B128" s="30"/>
-      <c r="C128" s="30"/>
-      <c r="D128" s="30"/>
-      <c r="E128" s="31"/>
-      <c r="F128" s="31"/>
-      <c r="G128" s="32"/>
-      <c r="H128" s="32"/>
-      <c r="I128" s="33"/>
+      <c r="B128" s="31"/>
+      <c r="C128" s="31"/>
+      <c r="D128" s="31"/>
+      <c r="E128" s="32"/>
+      <c r="F128" s="32"/>
+      <c r="G128" s="33"/>
+      <c r="H128" s="33"/>
+      <c r="I128" s="34"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="30"/>
-      <c r="B129" s="30"/>
-      <c r="C129" s="30"/>
-      <c r="D129" s="30"/>
-      <c r="E129" s="31"/>
-      <c r="F129" s="31"/>
-      <c r="G129" s="32"/>
-      <c r="H129" s="32"/>
-      <c r="I129" s="33"/>
+      <c r="B129" s="31"/>
+      <c r="C129" s="31"/>
+      <c r="D129" s="31"/>
+      <c r="E129" s="32"/>
+      <c r="F129" s="32"/>
+      <c r="G129" s="33"/>
+      <c r="H129" s="33"/>
+      <c r="I129" s="34"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="30"/>
-      <c r="B130" s="30"/>
-      <c r="C130" s="30"/>
-      <c r="D130" s="30"/>
-      <c r="E130" s="31"/>
-      <c r="F130" s="31"/>
-      <c r="G130" s="32"/>
-      <c r="H130" s="32"/>
-      <c r="I130" s="33"/>
+      <c r="B130" s="31"/>
+      <c r="C130" s="31"/>
+      <c r="D130" s="31"/>
+      <c r="E130" s="32"/>
+      <c r="F130" s="32"/>
+      <c r="G130" s="33"/>
+      <c r="H130" s="33"/>
+      <c r="I130" s="34"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="30"/>
-      <c r="B131" s="30"/>
-      <c r="C131" s="30"/>
-      <c r="D131" s="30"/>
-      <c r="E131" s="31"/>
-      <c r="F131" s="31"/>
-      <c r="G131" s="32"/>
-      <c r="H131" s="32"/>
-      <c r="I131" s="33"/>
+      <c r="B131" s="31"/>
+      <c r="C131" s="31"/>
+      <c r="D131" s="31"/>
+      <c r="E131" s="32"/>
+      <c r="F131" s="32"/>
+      <c r="G131" s="33"/>
+      <c r="H131" s="33"/>
+      <c r="I131" s="34"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="30"/>
-      <c r="B132" s="30"/>
-      <c r="C132" s="30"/>
-      <c r="D132" s="30"/>
-      <c r="E132" s="31"/>
-      <c r="F132" s="31"/>
-      <c r="G132" s="32"/>
-      <c r="H132" s="32"/>
-      <c r="I132" s="33"/>
+      <c r="B132" s="31"/>
+      <c r="C132" s="31"/>
+      <c r="D132" s="31"/>
+      <c r="E132" s="32"/>
+      <c r="F132" s="32"/>
+      <c r="G132" s="33"/>
+      <c r="H132" s="33"/>
+      <c r="I132" s="34"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="30"/>
-      <c r="B133" s="30"/>
-      <c r="C133" s="30"/>
-      <c r="D133" s="30"/>
-      <c r="E133" s="31"/>
-      <c r="F133" s="31"/>
-      <c r="G133" s="32"/>
-      <c r="H133" s="32"/>
-      <c r="I133" s="33"/>
+      <c r="B133" s="31"/>
+      <c r="C133" s="31"/>
+      <c r="D133" s="31"/>
+      <c r="E133" s="32"/>
+      <c r="F133" s="32"/>
+      <c r="G133" s="33"/>
+      <c r="H133" s="33"/>
+      <c r="I133" s="34"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="30"/>
-      <c r="B134" s="30"/>
-      <c r="C134" s="30"/>
-      <c r="D134" s="30"/>
-      <c r="E134" s="31"/>
-      <c r="F134" s="31"/>
-      <c r="G134" s="32"/>
-      <c r="H134" s="32"/>
-      <c r="I134" s="33"/>
+      <c r="B134" s="31"/>
+      <c r="C134" s="31"/>
+      <c r="D134" s="31"/>
+      <c r="E134" s="32"/>
+      <c r="F134" s="32"/>
+      <c r="G134" s="33"/>
+      <c r="H134" s="33"/>
+      <c r="I134" s="34"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="30"/>
-      <c r="B135" s="30"/>
-      <c r="C135" s="30"/>
-      <c r="D135" s="30"/>
-      <c r="E135" s="31"/>
-      <c r="F135" s="31"/>
-      <c r="G135" s="32"/>
-      <c r="H135" s="32"/>
-      <c r="I135" s="33"/>
+      <c r="B135" s="31"/>
+      <c r="C135" s="31"/>
+      <c r="D135" s="31"/>
+      <c r="E135" s="32"/>
+      <c r="F135" s="32"/>
+      <c r="G135" s="33"/>
+      <c r="H135" s="33"/>
+      <c r="I135" s="34"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="30"/>
-      <c r="B136" s="30"/>
-      <c r="C136" s="30"/>
-      <c r="D136" s="30"/>
-      <c r="E136" s="31"/>
-      <c r="F136" s="31"/>
-      <c r="G136" s="32"/>
-      <c r="H136" s="32"/>
-      <c r="I136" s="33"/>
+      <c r="B136" s="31"/>
+      <c r="C136" s="31"/>
+      <c r="D136" s="31"/>
+      <c r="E136" s="32"/>
+      <c r="F136" s="32"/>
+      <c r="G136" s="33"/>
+      <c r="H136" s="33"/>
+      <c r="I136" s="34"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="30"/>
-      <c r="B137" s="30"/>
-      <c r="C137" s="30"/>
-      <c r="D137" s="30"/>
-      <c r="E137" s="31"/>
-      <c r="F137" s="31"/>
-      <c r="G137" s="32"/>
-      <c r="H137" s="32"/>
-      <c r="I137" s="33"/>
+      <c r="B137" s="31"/>
+      <c r="C137" s="31"/>
+      <c r="D137" s="31"/>
+      <c r="E137" s="32"/>
+      <c r="F137" s="32"/>
+      <c r="G137" s="33"/>
+      <c r="H137" s="33"/>
+      <c r="I137" s="34"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="30"/>
-      <c r="B138" s="30"/>
-      <c r="C138" s="30"/>
-      <c r="D138" s="30"/>
-      <c r="E138" s="31"/>
-      <c r="F138" s="31"/>
-      <c r="G138" s="32"/>
-      <c r="H138" s="32"/>
-      <c r="I138" s="33"/>
+      <c r="B138" s="31"/>
+      <c r="C138" s="31"/>
+      <c r="D138" s="31"/>
+      <c r="E138" s="32"/>
+      <c r="F138" s="32"/>
+      <c r="G138" s="33"/>
+      <c r="H138" s="33"/>
+      <c r="I138" s="34"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="30"/>
-      <c r="B139" s="30"/>
-      <c r="C139" s="30"/>
-      <c r="D139" s="30"/>
-      <c r="E139" s="31"/>
-      <c r="F139" s="31"/>
-      <c r="G139" s="32"/>
-      <c r="H139" s="32"/>
-      <c r="I139" s="33"/>
+      <c r="B139" s="31"/>
+      <c r="C139" s="31"/>
+      <c r="D139" s="31"/>
+      <c r="E139" s="32"/>
+      <c r="F139" s="32"/>
+      <c r="G139" s="33"/>
+      <c r="H139" s="33"/>
+      <c r="I139" s="34"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="30"/>
-      <c r="B140" s="30"/>
-      <c r="C140" s="30"/>
-      <c r="D140" s="30"/>
-      <c r="E140" s="31"/>
-      <c r="F140" s="31"/>
-      <c r="G140" s="32"/>
-      <c r="H140" s="32"/>
-      <c r="I140" s="33"/>
+      <c r="B140" s="31"/>
+      <c r="C140" s="31"/>
+      <c r="D140" s="31"/>
+      <c r="E140" s="32"/>
+      <c r="F140" s="32"/>
+      <c r="G140" s="33"/>
+      <c r="H140" s="33"/>
+      <c r="I140" s="34"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="30"/>
-      <c r="B141" s="30"/>
-      <c r="C141" s="30"/>
-      <c r="D141" s="30"/>
-      <c r="E141" s="31"/>
-      <c r="F141" s="31"/>
-      <c r="G141" s="32"/>
-      <c r="H141" s="32"/>
-      <c r="I141" s="33"/>
+      <c r="B141" s="31"/>
+      <c r="C141" s="31"/>
+      <c r="D141" s="31"/>
+      <c r="E141" s="32"/>
+      <c r="F141" s="32"/>
+      <c r="G141" s="33"/>
+      <c r="H141" s="33"/>
+      <c r="I141" s="34"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="30"/>
-      <c r="B142" s="30"/>
-      <c r="C142" s="30"/>
-      <c r="D142" s="30"/>
-      <c r="E142" s="31"/>
-      <c r="F142" s="31"/>
-      <c r="G142" s="32"/>
-      <c r="H142" s="32"/>
-      <c r="I142" s="33"/>
+      <c r="B142" s="31"/>
+      <c r="C142" s="31"/>
+      <c r="D142" s="31"/>
+      <c r="E142" s="32"/>
+      <c r="F142" s="32"/>
+      <c r="G142" s="33"/>
+      <c r="H142" s="33"/>
+      <c r="I142" s="34"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="30"/>
-      <c r="B143" s="30"/>
-      <c r="C143" s="30"/>
-      <c r="D143" s="30"/>
-      <c r="E143" s="31"/>
-      <c r="F143" s="31"/>
-      <c r="G143" s="32"/>
-      <c r="H143" s="32"/>
-      <c r="I143" s="33"/>
+      <c r="B143" s="31"/>
+      <c r="C143" s="31"/>
+      <c r="D143" s="31"/>
+      <c r="E143" s="32"/>
+      <c r="F143" s="32"/>
+      <c r="G143" s="33"/>
+      <c r="H143" s="33"/>
+      <c r="I143" s="34"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="30"/>
-      <c r="B144" s="30"/>
-      <c r="C144" s="30"/>
-      <c r="D144" s="30"/>
-      <c r="E144" s="31"/>
-      <c r="F144" s="31"/>
-      <c r="G144" s="32"/>
-      <c r="H144" s="32"/>
-      <c r="I144" s="33"/>
+      <c r="B144" s="31"/>
+      <c r="C144" s="31"/>
+      <c r="D144" s="31"/>
+      <c r="E144" s="32"/>
+      <c r="F144" s="32"/>
+      <c r="G144" s="33"/>
+      <c r="H144" s="33"/>
+      <c r="I144" s="34"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="30"/>
-      <c r="B145" s="30"/>
-      <c r="C145" s="30"/>
-      <c r="D145" s="30"/>
-      <c r="E145" s="31"/>
-      <c r="F145" s="31"/>
-      <c r="G145" s="32"/>
-      <c r="H145" s="32"/>
-      <c r="I145" s="33"/>
+      <c r="B145" s="31"/>
+      <c r="C145" s="31"/>
+      <c r="D145" s="31"/>
+      <c r="E145" s="32"/>
+      <c r="F145" s="32"/>
+      <c r="G145" s="33"/>
+      <c r="H145" s="33"/>
+      <c r="I145" s="34"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="30"/>
-      <c r="B146" s="30"/>
-      <c r="C146" s="30"/>
-      <c r="D146" s="30"/>
-      <c r="E146" s="31"/>
-      <c r="F146" s="31"/>
-      <c r="G146" s="32"/>
-      <c r="H146" s="32"/>
-      <c r="I146" s="33"/>
+      <c r="B146" s="31"/>
+      <c r="C146" s="31"/>
+      <c r="D146" s="31"/>
+      <c r="E146" s="32"/>
+      <c r="F146" s="32"/>
+      <c r="G146" s="33"/>
+      <c r="H146" s="33"/>
+      <c r="I146" s="34"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="30"/>
-      <c r="B147" s="30"/>
-      <c r="C147" s="30"/>
-      <c r="D147" s="30"/>
-      <c r="E147" s="31"/>
-      <c r="F147" s="31"/>
-      <c r="G147" s="32"/>
-      <c r="H147" s="32"/>
-      <c r="I147" s="33"/>
+      <c r="B147" s="31"/>
+      <c r="C147" s="31"/>
+      <c r="D147" s="31"/>
+      <c r="E147" s="32"/>
+      <c r="F147" s="32"/>
+      <c r="G147" s="33"/>
+      <c r="H147" s="33"/>
+      <c r="I147" s="34"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="30"/>
-      <c r="B148" s="30"/>
-      <c r="C148" s="30"/>
-      <c r="D148" s="30"/>
-      <c r="E148" s="31"/>
-      <c r="F148" s="31"/>
-      <c r="G148" s="32"/>
-      <c r="H148" s="32"/>
-      <c r="I148" s="33"/>
+      <c r="B148" s="31"/>
+      <c r="C148" s="31"/>
+      <c r="D148" s="31"/>
+      <c r="E148" s="32"/>
+      <c r="F148" s="32"/>
+      <c r="G148" s="33"/>
+      <c r="H148" s="33"/>
+      <c r="I148" s="34"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="30"/>
-      <c r="B149" s="30"/>
-      <c r="C149" s="30"/>
-      <c r="D149" s="30"/>
-      <c r="E149" s="31"/>
-      <c r="F149" s="31"/>
-      <c r="G149" s="32"/>
-      <c r="H149" s="32"/>
-      <c r="I149" s="33"/>
+      <c r="B149" s="31"/>
+      <c r="C149" s="31"/>
+      <c r="D149" s="31"/>
+      <c r="E149" s="32"/>
+      <c r="F149" s="32"/>
+      <c r="G149" s="33"/>
+      <c r="H149" s="33"/>
+      <c r="I149" s="34"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="30"/>
-      <c r="B150" s="30"/>
-      <c r="C150" s="30"/>
-      <c r="D150" s="30"/>
-      <c r="E150" s="31"/>
-      <c r="F150" s="31"/>
-      <c r="G150" s="32"/>
-      <c r="H150" s="32"/>
-      <c r="I150" s="33"/>
+      <c r="B150" s="31"/>
+      <c r="C150" s="31"/>
+      <c r="D150" s="31"/>
+      <c r="E150" s="32"/>
+      <c r="F150" s="32"/>
+      <c r="G150" s="33"/>
+      <c r="H150" s="33"/>
+      <c r="I150" s="34"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="30"/>
-      <c r="B151" s="30"/>
-      <c r="C151" s="30"/>
-      <c r="D151" s="30"/>
-      <c r="E151" s="31"/>
-      <c r="F151" s="31"/>
-      <c r="G151" s="32"/>
-      <c r="H151" s="32"/>
-      <c r="I151" s="33"/>
+      <c r="B151" s="31"/>
+      <c r="C151" s="31"/>
+      <c r="D151" s="31"/>
+      <c r="E151" s="32"/>
+      <c r="F151" s="32"/>
+      <c r="G151" s="33"/>
+      <c r="H151" s="33"/>
+      <c r="I151" s="34"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="30"/>
-      <c r="B152" s="30"/>
-      <c r="C152" s="30"/>
-      <c r="D152" s="30"/>
-      <c r="E152" s="31"/>
-      <c r="F152" s="31"/>
-      <c r="G152" s="32"/>
-      <c r="H152" s="32"/>
-      <c r="I152" s="33"/>
+      <c r="B152" s="31"/>
+      <c r="C152" s="31"/>
+      <c r="D152" s="31"/>
+      <c r="E152" s="32"/>
+      <c r="F152" s="32"/>
+      <c r="G152" s="33"/>
+      <c r="H152" s="33"/>
+      <c r="I152" s="34"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="30"/>
-      <c r="B153" s="30"/>
-      <c r="C153" s="30"/>
-      <c r="D153" s="30"/>
-      <c r="E153" s="31"/>
-      <c r="F153" s="31"/>
-      <c r="G153" s="32"/>
-      <c r="H153" s="32"/>
-      <c r="I153" s="33"/>
+      <c r="B153" s="31"/>
+      <c r="C153" s="31"/>
+      <c r="D153" s="31"/>
+      <c r="E153" s="32"/>
+      <c r="F153" s="32"/>
+      <c r="G153" s="33"/>
+      <c r="H153" s="33"/>
+      <c r="I153" s="34"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="30"/>
-      <c r="B154" s="30"/>
-      <c r="C154" s="30"/>
-      <c r="D154" s="30"/>
-      <c r="E154" s="31"/>
-      <c r="F154" s="31"/>
-      <c r="G154" s="32"/>
-      <c r="H154" s="32"/>
-      <c r="I154" s="33"/>
+      <c r="B154" s="31"/>
+      <c r="C154" s="31"/>
+      <c r="D154" s="31"/>
+      <c r="E154" s="32"/>
+      <c r="F154" s="32"/>
+      <c r="G154" s="33"/>
+      <c r="H154" s="33"/>
+      <c r="I154" s="34"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="30"/>
-      <c r="B155" s="30"/>
-      <c r="C155" s="30"/>
-      <c r="D155" s="30"/>
-      <c r="E155" s="31"/>
-      <c r="F155" s="31"/>
-      <c r="G155" s="32"/>
-      <c r="H155" s="32"/>
-      <c r="I155" s="33"/>
+      <c r="B155" s="31"/>
+      <c r="C155" s="31"/>
+      <c r="D155" s="31"/>
+      <c r="E155" s="32"/>
+      <c r="F155" s="32"/>
+      <c r="G155" s="33"/>
+      <c r="H155" s="33"/>
+      <c r="I155" s="34"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="30"/>
-      <c r="B156" s="30"/>
-      <c r="C156" s="30"/>
-      <c r="D156" s="30"/>
-      <c r="E156" s="31"/>
-      <c r="F156" s="31"/>
-      <c r="G156" s="32"/>
-      <c r="H156" s="32"/>
-      <c r="I156" s="33"/>
+      <c r="B156" s="31"/>
+      <c r="C156" s="31"/>
+      <c r="D156" s="31"/>
+      <c r="E156" s="32"/>
+      <c r="F156" s="32"/>
+      <c r="G156" s="33"/>
+      <c r="H156" s="33"/>
+      <c r="I156" s="34"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" error="Bitte IoT, EDM, Parking oder LLM auswählen." errorStyle="stop" errorTitle="Ungültiges Themenfeld" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A7:A356" type="list">
+    <dataValidation allowBlank="true" error="Bitte IoT, EDM, Parking oder LLM auswählen." errorStyle="stop" errorTitle="Ungültiges Themenfeld" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B356" type="list">
       <formula1>"IoT,EDM,Parking,LLM"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Bitte Hardware, Hardware + Dienstleistung, Lizenzen oder Dienstleistung auswählen." errorStyle="stop" errorTitle="Ungültige Kategorie" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B356" type="list">
+    <dataValidation allowBlank="true" error="Bitte Hardware, Hardware + Dienstleistung, Lizenzen oder Dienstleistung auswählen." errorStyle="stop" errorTitle="Ungültige Kategorie" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C7:C356" type="list">
       <formula1>"Hardware,Hardware + Dienstleistung,Lizenzen,Dienstleistung"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -19418,7 +19423,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="35" t="s">
         <v>93</v>
       </c>
     </row>
@@ -19428,21 +19433,21 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="37" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="38" t="s">
         <v>97</v>
       </c>
       <c r="B6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="39" t="s">
         <v>98</v>
       </c>
       <c r="B7" s="11" t="n">
@@ -19451,7 +19456,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="39" t="s">
         <v>99</v>
       </c>
       <c r="B8" s="11" t="n">
@@ -19460,7 +19465,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="40" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="23" t="n">
@@ -19469,13 +19474,13 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="38" t="s">
         <v>101</v>
       </c>
       <c r="B10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="39" t="s">
         <v>102</v>
       </c>
       <c r="B11" s="11" t="n">
@@ -19484,7 +19489,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="39" t="s">
         <v>103</v>
       </c>
       <c r="B12" s="11" t="n">
@@ -19493,7 +19498,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="40" t="s">
         <v>104</v>
       </c>
       <c r="B13" s="23" t="n">
@@ -19502,13 +19507,13 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="38" t="s">
         <v>105</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="39" t="s">
         <v>106</v>
       </c>
       <c r="B15" s="11" t="n">
@@ -19517,7 +19522,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="39" t="s">
         <v>107</v>
       </c>
       <c r="B16" s="11" t="n">
@@ -19526,7 +19531,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="40" t="s">
         <v>108</v>
       </c>
       <c r="B17" s="23" t="n">

</xml_diff>